<commit_message>
Docs HTML : règlements, plan questionnaire, guide rédaction + refonte nav
- Nouvelles pages HTML : reglements.html, plan-questionnaire.html,
  guide-redaction.html (thème clair, nav identique aux pages stats)
- docs.html : refonte thème clair, ajout nav avec dropdown Ressources,
  liens "Consulter" vers les pages HTML (au lieu de téléchargement direct),
  ajout Procès-verbaux et Plan du questionnaire
- Toutes les pages stats + docs : remplacement des liens épars par un
  dropdown "Ressources" (Documentation + Saisons précédentes),
  suppression du lien "Feuille de match" de la nav principale
- Fichiers ressources : gabarit-q3.xlsx (v2.1 saison 2025-2026),
  reglements.doc, plan-questionnaire.doc, guide-redaction.doc

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/ressources/2025-2026/gabarit-q3.xlsx
+++ b/public/ressources/2025-2026/gabarit-q3.xlsx
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="148">
   <si>
     <r>
       <rPr>
@@ -280,7 +280,10 @@
     <t xml:space="preserve">Sous-thème 1 (doit être précis et non relié au sous-thème 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">st13.a</t>
+    <t xml:space="preserve">Saisir sous-thème 1 ici</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saisir question thème 1 ici</t>
   </si>
   <si>
     <t xml:space="preserve">A</t>
@@ -298,7 +301,10 @@
     <t xml:space="preserve">Sous-thème 2 (doit être précis et non relié au sous-thème 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">st13.b</t>
+    <t xml:space="preserve">Saisir sous-thème 2 ici</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saisir question thème 2 ici</t>
   </si>
   <si>
     <t xml:space="preserve">Série 14</t>
@@ -350,6 +356,12 @@
   </si>
   <si>
     <t xml:space="preserve">Réponse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2</t>
   </si>
   <si>
     <t xml:space="preserve">28 mars 2003</t>
@@ -744,8 +756,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
+      <i val="true"/>
       <sz val="12"/>
+      <color rgb="FF808080"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
@@ -838,7 +851,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="56">
+  <borders count="54">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1107,36 +1120,15 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
       <right style="medium"/>
       <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
       <right style="thin"/>
       <top/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
       <bottom style="medium"/>
       <diagonal/>
     </border>
@@ -1213,6 +1205,13 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
       <right style="thin"/>
       <top style="thin"/>
       <bottom/>
@@ -1276,7 +1275,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="128">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1581,11 +1580,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1593,7 +1588,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1601,11 +1596,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -1621,15 +1612,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1641,7 +1624,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="41" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -1653,7 +1636,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="45" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="42" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1693,35 +1676,35 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="46" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="43" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="46" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="43" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1729,23 +1712,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1753,55 +1736,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="49" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="46" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="50" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="47" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="48" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="49" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="50" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="47" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="51" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="38" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="52" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="50" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="52" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="53" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="54" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="54" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="55" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1817,13 +1800,34 @@
     <cellStyle name="Normal_Auteur" xfId="21"/>
     <cellStyle name="Normal_Vers BD" xfId="22"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <font>
         <name val="Arial"/>
         <charset val="1"/>
         <family val="0"/>
       </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="10"/>
+        <u val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="General"/>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
@@ -1845,9 +1849,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2522160</xdr:colOff>
+      <xdr:colOff>2521080</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>122040</xdr:rowOff>
+      <xdr:rowOff>120960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1857,7 +1861,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="681840" y="325800"/>
-          <a:ext cx="2715840" cy="1443960"/>
+          <a:ext cx="2714760" cy="1442880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1997,9 +2001,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>468720</xdr:colOff>
+      <xdr:colOff>467640</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>179280</xdr:rowOff>
+      <xdr:rowOff>178200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2009,7 +2013,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9114120" y="314280"/>
-          <a:ext cx="1581120" cy="369720"/>
+          <a:ext cx="1580040" cy="368640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2069,7 +2073,7 @@
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>Version 2.0</a:t>
+            <a:t>Version 2.1</a:t>
           </a:r>
           <a:endParaRPr lang="fr-CA" sz="1000" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -2090,9 +2094,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2160</xdr:colOff>
+      <xdr:colOff>1080</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>181080</xdr:rowOff>
+      <xdr:rowOff>180000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2102,7 +2106,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="478080"/>
-          <a:ext cx="636480" cy="1350720"/>
+          <a:ext cx="635400" cy="1349640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2473,9 +2477,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="6"/>
-      <c r="D2" s="7" t="n">
-        <v>3</v>
-      </c>
+      <c r="D2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="6" t="s">
@@ -3652,8 +3654,8 @@
         <v>50</v>
       </c>
       <c r="D125" s="16" t="str">
-        <f aca="false">C129 &amp; " / " &amp; C140</f>
-        <v>st13.a / st13.b</v>
+        <f aca="false">C128 &amp; " / " &amp;C139</f>
+        <v>Saisir sous-thème 1 ici / Saisir sous-thème 2 ici</v>
       </c>
       <c r="E125" s="23"/>
     </row>
@@ -3667,26 +3669,26 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="75"/>
-      <c r="C127" s="76" t="s">
+      <c r="C127" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="D127" s="77"/>
+      <c r="D127" s="76"/>
       <c r="E127" s="23"/>
     </row>
-    <row r="128" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B128" s="78"/>
-      <c r="C128" s="79" t="s">
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B128" s="77"/>
+      <c r="C128" s="78" t="s">
         <v>53</v>
       </c>
-      <c r="D128" s="80"/>
+      <c r="D128" s="79"/>
       <c r="E128" s="23"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B129" s="81"/>
-      <c r="C129" s="79" t="s">
-        <v>53</v>
-      </c>
-      <c r="D129" s="80"/>
+      <c r="B129" s="77"/>
+      <c r="C129" s="78" t="s">
+        <v>54</v>
+      </c>
+      <c r="D129" s="79"/>
       <c r="E129" s="23"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3729,64 +3731,64 @@
       <c r="B133" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="C133" s="82"/>
+      <c r="C133" s="80"/>
       <c r="D133" s="27"/>
       <c r="E133" s="23"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B134" s="83" t="s">
-        <v>54</v>
+      <c r="B134" s="81" t="s">
+        <v>55</v>
       </c>
       <c r="C134" s="71"/>
       <c r="D134" s="72"/>
       <c r="E134" s="23"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B135" s="84" t="s">
-        <v>55</v>
+      <c r="B135" s="82" t="s">
+        <v>56</v>
       </c>
       <c r="C135" s="32"/>
       <c r="D135" s="22"/>
       <c r="E135" s="23"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B136" s="84" t="s">
-        <v>56</v>
+      <c r="B136" s="82" t="s">
+        <v>57</v>
       </c>
       <c r="C136" s="32"/>
       <c r="D136" s="22"/>
       <c r="E136" s="23"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B137" s="85" t="s">
-        <v>57</v>
+      <c r="B137" s="83" t="s">
+        <v>58</v>
       </c>
       <c r="C137" s="26"/>
       <c r="D137" s="27"/>
       <c r="E137" s="23"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B138" s="78"/>
-      <c r="C138" s="86" t="s">
-        <v>58</v>
-      </c>
-      <c r="D138" s="80"/>
+      <c r="B138" s="77"/>
+      <c r="C138" s="45" t="s">
+        <v>59</v>
+      </c>
+      <c r="D138" s="79"/>
       <c r="E138" s="23"/>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B139" s="78"/>
-      <c r="C139" s="86" t="s">
-        <v>59</v>
-      </c>
-      <c r="D139" s="80"/>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B139" s="77"/>
+      <c r="C139" s="78" t="s">
+        <v>60</v>
+      </c>
+      <c r="D139" s="79"/>
       <c r="E139" s="23"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B140" s="81"/>
-      <c r="C140" s="87" t="s">
-        <v>59</v>
-      </c>
-      <c r="D140" s="88"/>
+      <c r="B140" s="77"/>
+      <c r="C140" s="78" t="s">
+        <v>61</v>
+      </c>
+      <c r="D140" s="84"/>
       <c r="E140" s="23"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3829,62 +3831,62 @@
       <c r="B144" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="C144" s="82"/>
+      <c r="C144" s="80"/>
       <c r="D144" s="27"/>
       <c r="E144" s="23"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B145" s="83" t="s">
-        <v>54</v>
+      <c r="B145" s="81" t="s">
+        <v>55</v>
       </c>
       <c r="C145" s="71"/>
       <c r="D145" s="72"/>
       <c r="E145" s="23"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B146" s="84" t="s">
-        <v>55</v>
+      <c r="B146" s="82" t="s">
+        <v>56</v>
       </c>
       <c r="C146" s="32"/>
       <c r="D146" s="22"/>
       <c r="E146" s="23"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B147" s="84" t="s">
-        <v>56</v>
+      <c r="B147" s="82" t="s">
+        <v>57</v>
       </c>
       <c r="C147" s="32"/>
       <c r="D147" s="22"/>
       <c r="E147" s="23"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B148" s="85" t="s">
-        <v>57</v>
+      <c r="B148" s="83" t="s">
+        <v>58</v>
       </c>
       <c r="C148" s="26"/>
       <c r="D148" s="27"/>
       <c r="E148" s="23"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B149" s="89"/>
-      <c r="C149" s="89"/>
-      <c r="D149" s="90"/>
+      <c r="B149" s="85"/>
+      <c r="C149" s="85"/>
+      <c r="D149" s="86"/>
       <c r="E149" s="23"/>
     </row>
     <row r="150" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B150" s="11"/>
       <c r="C150" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D150" s="13" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E150" s="23"/>
     </row>
     <row r="151" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B151" s="14"/>
       <c r="C151" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D151" s="16"/>
       <c r="E151" s="23"/>
@@ -3892,7 +3894,7 @@
     <row r="152" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B152" s="29"/>
       <c r="C152" s="17" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D152" s="18"/>
       <c r="E152" s="23"/>
@@ -4003,8 +4005,8 @@
       <c r="B162" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="C162" s="82"/>
-      <c r="D162" s="91"/>
+      <c r="C162" s="80"/>
+      <c r="D162" s="87"/>
       <c r="E162" s="23"/>
     </row>
     <row r="163" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4016,17 +4018,17 @@
     <row r="164" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B164" s="11"/>
       <c r="C164" s="12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D164" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E164" s="23"/>
     </row>
     <row r="165" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B165" s="14"/>
       <c r="C165" s="15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D165" s="16"/>
       <c r="E165" s="23"/>
@@ -4034,7 +4036,7 @@
     <row r="166" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B166" s="29"/>
       <c r="C166" s="17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D166" s="18"/>
       <c r="E166" s="23"/>
@@ -4084,6 +4086,11 @@
       <formula>NOT(ISERROR(SEARCH("-- Choisir un thème --",D60)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D2">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D60" type="list">
       <formula1>"-- Choisir un thème --,Arts et littérature,Cinéma et télévision,Musique"</formula1>
@@ -4093,12 +4100,12 @@
       <formula1>"-- Choisir un thème --,Actualité,Histoire et société,Langue"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D124" type="list">
+    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D91" type="list">
       <formula1>"-- Choisir un thème --,Actualité,Arts et littérature,Cinéma et télévision,Géographie,Histoire et société,Langue,Musique,Sciences,Sports et loisirs"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D91" type="list">
-      <formula1>"-- Choisir un thème --,Actualité,Arts et littérature,Cinéma et télévision,Géographie,Histoire et société,Langue,Musique,Sciences,Sports et loisirs"</formula1>
+    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D124" type="list">
+      <formula1>"-- Choisir un thème --,Divers,Actualité,Arts et littérature,Cinéma et télévision,Géographie,Histoire et société,Langue,Musique,Sciences,Sports et loisirs"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4124,14 +4131,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:IT109"/>
+  <dimension ref="A1:IT111"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="14.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="7.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="22.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="52.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="28.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="34.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="14.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="7.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="6.57"/>
@@ -4140,28 +4147,28 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="92" t="s">
-        <v>68</v>
+      <c r="A1" s="88" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="93" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="93" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="93" t="s">
+      <c r="A2" s="89" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="93" t="s">
+      <c r="B2" s="89" t="s">
         <v>72</v>
+      </c>
+      <c r="C2" s="89" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="89" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>1</v>
@@ -4178,7 +4185,7 @@
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">B3+1</f>
@@ -4192,15 +4199,15 @@
         <f aca="true">IF(INDIRECT(Adresses!E17)&lt;&gt;0,INDIRECT(Adresses!E17),"")</f>
         <v/>
       </c>
-      <c r="F4" s="94"/>
-      <c r="G4" s="94"/>
-      <c r="H4" s="94"/>
-      <c r="I4" s="94"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B5" s="2" t="n">
         <f aca="false">B4+1</f>
@@ -4218,7 +4225,7 @@
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">B5+1</f>
@@ -4236,7 +4243,7 @@
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B7" s="2" t="n">
         <f aca="false">B6+1</f>
@@ -4254,7 +4261,7 @@
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B8" s="2" t="n">
         <f aca="false">B7+1</f>
@@ -4272,7 +4279,7 @@
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B9" s="2" t="n">
         <f aca="false">B8+1</f>
@@ -4290,7 +4297,7 @@
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B10" s="2" t="n">
         <f aca="false">B9+1</f>
@@ -4308,7 +4315,7 @@
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B11" s="2" t="n">
         <f aca="false">B10+1</f>
@@ -4326,7 +4333,7 @@
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B12" s="2" t="n">
         <f aca="false">B11+1</f>
@@ -4344,7 +4351,7 @@
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B13" s="2" t="n">
         <f aca="false">B12+1</f>
@@ -4362,7 +4369,7 @@
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B14" s="2" t="n">
         <f aca="false">B13+1</f>
@@ -4380,7 +4387,7 @@
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B15" s="2" t="n">
         <f aca="false">B14+1</f>
@@ -4392,13 +4399,13 @@
       </c>
       <c r="D15" s="2" t="str">
         <f aca="true">IF(INDIRECT(Adresses!E72)&lt;&gt;0,INDIRECT(Adresses!E72),"")</f>
-        <v>st13.a / st13.b</v>
+        <v>Saisir sous-thème 1 ici / Saisir sous-thème 2 ici</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B16" s="2" t="n">
         <f aca="false">B15+1</f>
@@ -4416,7 +4423,7 @@
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B17" s="2" t="n">
         <f aca="false">B16+1</f>
@@ -4432,44 +4439,44 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="92" t="s">
-        <v>73</v>
+      <c r="A19" s="88" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="93" t="s">
-        <v>69</v>
-      </c>
-      <c r="B20" s="93" t="s">
-        <v>70</v>
-      </c>
-      <c r="C20" s="93" t="s">
-        <v>74</v>
-      </c>
-      <c r="D20" s="93" t="s">
-        <v>75</v>
-      </c>
-      <c r="E20" s="93" t="s">
+      <c r="A20" s="89" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="89" t="s">
         <v>76</v>
+      </c>
+      <c r="D20" s="89" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="89" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B21" s="94" t="n">
+        <v>0</v>
+      </c>
+      <c r="B21" s="90" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="94" t="n">
+      <c r="C21" s="90" t="n">
         <f aca="false">Auteur!B14</f>
         <v>1</v>
       </c>
-      <c r="D21" s="94" t="n">
+      <c r="D21" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G9)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="94" t="n">
+      <c r="E21" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H9)</f>
         <v>0</v>
       </c>
@@ -4477,20 +4484,20 @@
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="94" t="n">
+      <c r="C22" s="90" t="n">
         <f aca="false">Auteur!B15</f>
         <v>2</v>
       </c>
-      <c r="D22" s="94" t="n">
+      <c r="D22" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G10)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="94" t="n">
+      <c r="E22" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H10)</f>
         <v>0</v>
       </c>
@@ -4498,20 +4505,20 @@
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="94" t="n">
+      <c r="C23" s="90" t="n">
         <f aca="false">Auteur!B16</f>
         <v>3</v>
       </c>
-      <c r="D23" s="94" t="n">
+      <c r="D23" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G11)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="94" t="n">
+      <c r="E23" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H11)</f>
         <v>0</v>
       </c>
@@ -4519,20 +4526,20 @@
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="94" t="n">
+      <c r="C24" s="90" t="n">
         <f aca="false">Auteur!B17</f>
         <v>4</v>
       </c>
-      <c r="D24" s="94" t="n">
+      <c r="D24" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G12)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="94" t="n">
+      <c r="E24" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H12)</f>
         <v>0</v>
       </c>
@@ -4540,20 +4547,20 @@
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C25" s="94" t="n">
+      <c r="C25" s="90" t="n">
         <f aca="false">Auteur!B19</f>
         <v>5</v>
       </c>
-      <c r="D25" s="94" t="n">
+      <c r="D25" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G13)</f>
         <v>0</v>
       </c>
-      <c r="E25" s="94" t="n">
+      <c r="E25" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H13)</f>
         <v>0</v>
       </c>
@@ -4561,20 +4568,20 @@
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C26" s="94" t="n">
+      <c r="C26" s="90" t="n">
         <f aca="false">Auteur!B20</f>
         <v>6</v>
       </c>
-      <c r="D26" s="94" t="n">
+      <c r="D26" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G14)</f>
         <v>0</v>
       </c>
-      <c r="E26" s="94" t="n">
+      <c r="E26" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H14)</f>
         <v>0</v>
       </c>
@@ -4582,20 +4589,20 @@
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C27" s="94" t="n">
+      <c r="C27" s="90" t="n">
         <f aca="false">Auteur!B21</f>
         <v>7</v>
       </c>
-      <c r="D27" s="94" t="n">
+      <c r="D27" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G15)</f>
         <v>0</v>
       </c>
-      <c r="E27" s="94" t="n">
+      <c r="E27" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H15)</f>
         <v>0</v>
       </c>
@@ -4603,20 +4610,20 @@
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C28" s="94" t="n">
+      <c r="C28" s="90" t="n">
         <f aca="false">Auteur!B22</f>
         <v>8</v>
       </c>
-      <c r="D28" s="94" t="n">
+      <c r="D28" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G16)</f>
         <v>0</v>
       </c>
-      <c r="E28" s="94" t="n">
+      <c r="E28" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H16)</f>
         <v>0</v>
       </c>
@@ -4624,20 +4631,20 @@
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C29" s="94" t="n">
+      <c r="C29" s="90" t="n">
         <f aca="false">Auteur!B27</f>
         <v>1</v>
       </c>
-      <c r="D29" s="94" t="n">
+      <c r="D29" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G17)</f>
         <v>0</v>
       </c>
-      <c r="E29" s="94" t="n">
+      <c r="E29" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H17)</f>
         <v>0</v>
       </c>
@@ -4645,20 +4652,20 @@
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C30" s="94" t="n">
+      <c r="C30" s="90" t="n">
         <f aca="false">Auteur!B28</f>
         <v>2</v>
       </c>
-      <c r="D30" s="94" t="n">
+      <c r="D30" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G18)</f>
         <v>0</v>
       </c>
-      <c r="E30" s="94" t="n">
+      <c r="E30" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H18)</f>
         <v>0</v>
       </c>
@@ -4666,20 +4673,20 @@
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C31" s="94" t="n">
+      <c r="C31" s="90" t="n">
         <f aca="false">Auteur!B29</f>
         <v>3</v>
       </c>
-      <c r="D31" s="94" t="n">
+      <c r="D31" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G19)</f>
         <v>0</v>
       </c>
-      <c r="E31" s="94" t="n">
+      <c r="E31" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H19)</f>
         <v>0</v>
       </c>
@@ -4687,20 +4694,20 @@
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="94" t="n">
+      <c r="C32" s="90" t="n">
         <f aca="false">Auteur!B30</f>
         <v>4</v>
       </c>
-      <c r="D32" s="94" t="n">
+      <c r="D32" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G20)</f>
         <v>0</v>
       </c>
-      <c r="E32" s="94" t="n">
+      <c r="E32" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H20)</f>
         <v>0</v>
       </c>
@@ -4708,20 +4715,20 @@
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C33" s="94" t="n">
+      <c r="C33" s="90" t="n">
         <f aca="false">Auteur!B31</f>
         <v>5</v>
       </c>
-      <c r="D33" s="94" t="n">
+      <c r="D33" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G21)</f>
         <v>0</v>
       </c>
-      <c r="E33" s="94" t="n">
+      <c r="E33" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H21)</f>
         <v>0</v>
       </c>
@@ -4729,20 +4736,20 @@
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C34" s="94" t="n">
+      <c r="C34" s="90" t="n">
         <f aca="false">Auteur!B36</f>
         <v>1</v>
       </c>
-      <c r="D34" s="94" t="n">
+      <c r="D34" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G22)</f>
         <v>0</v>
       </c>
-      <c r="E34" s="94" t="n">
+      <c r="E34" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H22)</f>
         <v>0</v>
       </c>
@@ -4750,20 +4757,20 @@
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C35" s="94" t="n">
+      <c r="C35" s="90" t="n">
         <f aca="false">Auteur!B37</f>
         <v>2</v>
       </c>
-      <c r="D35" s="94" t="n">
+      <c r="D35" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G23)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="94" t="n">
+      <c r="E35" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H23)</f>
         <v>0</v>
       </c>
@@ -4771,20 +4778,20 @@
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C36" s="94" t="n">
+      <c r="C36" s="90" t="n">
         <f aca="false">Auteur!B38</f>
         <v>3</v>
       </c>
-      <c r="D36" s="94" t="n">
+      <c r="D36" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G24)</f>
         <v>0</v>
       </c>
-      <c r="E36" s="94" t="n">
+      <c r="E36" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H24)</f>
         <v>0</v>
       </c>
@@ -4792,20 +4799,20 @@
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C37" s="94" t="n">
+      <c r="C37" s="90" t="n">
         <f aca="false">Auteur!B39</f>
         <v>4</v>
       </c>
-      <c r="D37" s="94" t="n">
+      <c r="D37" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G25)</f>
         <v>0</v>
       </c>
-      <c r="E37" s="94" t="n">
+      <c r="E37" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H25)</f>
         <v>0</v>
       </c>
@@ -4813,20 +4820,20 @@
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C38" s="94" t="n">
+      <c r="C38" s="90" t="n">
         <f aca="false">Auteur!B40</f>
         <v>5</v>
       </c>
-      <c r="D38" s="94" t="n">
+      <c r="D38" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G26)</f>
         <v>0</v>
       </c>
-      <c r="E38" s="94" t="n">
+      <c r="E38" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H26)</f>
         <v>0</v>
       </c>
@@ -4834,20 +4841,20 @@
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C39" s="94" t="n">
+      <c r="C39" s="90" t="n">
         <f aca="false">Auteur!B45</f>
         <v>1</v>
       </c>
-      <c r="D39" s="94" t="n">
+      <c r="D39" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G27)</f>
         <v>0</v>
       </c>
-      <c r="E39" s="94" t="n">
+      <c r="E39" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H27)</f>
         <v>0</v>
       </c>
@@ -4855,20 +4862,20 @@
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C40" s="94" t="n">
+      <c r="C40" s="90" t="n">
         <f aca="false">Auteur!B46</f>
         <v>2</v>
       </c>
-      <c r="D40" s="94" t="n">
+      <c r="D40" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G28)</f>
         <v>0</v>
       </c>
-      <c r="E40" s="94" t="n">
+      <c r="E40" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H28)</f>
         <v>0</v>
       </c>
@@ -4876,20 +4883,20 @@
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C41" s="94" t="n">
+      <c r="C41" s="90" t="n">
         <f aca="false">Auteur!B47</f>
         <v>3</v>
       </c>
-      <c r="D41" s="94" t="n">
+      <c r="D41" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G29)</f>
         <v>0</v>
       </c>
-      <c r="E41" s="94" t="n">
+      <c r="E41" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H29)</f>
         <v>0</v>
       </c>
@@ -4897,20 +4904,20 @@
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C42" s="94" t="n">
+      <c r="C42" s="90" t="n">
         <f aca="false">Auteur!B48</f>
         <v>4</v>
       </c>
-      <c r="D42" s="94" t="n">
+      <c r="D42" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G30)</f>
         <v>0</v>
       </c>
-      <c r="E42" s="94" t="n">
+      <c r="E42" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H30)</f>
         <v>0</v>
       </c>
@@ -4918,20 +4925,20 @@
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C43" s="94" t="n">
+      <c r="C43" s="90" t="n">
         <f aca="false">Auteur!B49</f>
         <v>5</v>
       </c>
-      <c r="D43" s="94" t="n">
+      <c r="D43" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G31)</f>
         <v>0</v>
       </c>
-      <c r="E43" s="94" t="n">
+      <c r="E43" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H31)</f>
         <v>0</v>
       </c>
@@ -4939,20 +4946,20 @@
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C44" s="94" t="n">
+      <c r="C44" s="90" t="n">
         <f aca="false">Auteur!B54</f>
         <v>1</v>
       </c>
-      <c r="D44" s="94" t="n">
+      <c r="D44" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G32)</f>
         <v>0</v>
       </c>
-      <c r="E44" s="94" t="n">
+      <c r="E44" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H32)</f>
         <v>0</v>
       </c>
@@ -4960,20 +4967,20 @@
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C45" s="94" t="n">
+      <c r="C45" s="90" t="n">
         <f aca="false">Auteur!B55</f>
         <v>2</v>
       </c>
-      <c r="D45" s="94" t="n">
+      <c r="D45" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G33)</f>
         <v>0</v>
       </c>
-      <c r="E45" s="94" t="n">
+      <c r="E45" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H33)</f>
         <v>0</v>
       </c>
@@ -4981,20 +4988,20 @@
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C46" s="94" t="n">
+      <c r="C46" s="90" t="n">
         <f aca="false">Auteur!B56</f>
         <v>3</v>
       </c>
-      <c r="D46" s="94" t="n">
+      <c r="D46" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G34)</f>
         <v>0</v>
       </c>
-      <c r="E46" s="94" t="n">
+      <c r="E46" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H34)</f>
         <v>0</v>
       </c>
@@ -5002,20 +5009,20 @@
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C47" s="94" t="n">
+      <c r="C47" s="90" t="n">
         <f aca="false">Auteur!B57</f>
         <v>4</v>
       </c>
-      <c r="D47" s="94" t="n">
+      <c r="D47" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G35)</f>
         <v>0</v>
       </c>
-      <c r="E47" s="94" t="n">
+      <c r="E47" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H35)</f>
         <v>0</v>
       </c>
@@ -5023,20 +5030,20 @@
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C48" s="94" t="n">
+      <c r="C48" s="90" t="n">
         <f aca="false">Auteur!B58</f>
         <v>5</v>
       </c>
-      <c r="D48" s="94" t="n">
+      <c r="D48" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G36)</f>
         <v>0</v>
       </c>
-      <c r="E48" s="94" t="n">
+      <c r="E48" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H36)</f>
         <v>0</v>
       </c>
@@ -5044,20 +5051,20 @@
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C49" s="94" t="n">
+      <c r="C49" s="90" t="n">
         <f aca="false">Auteur!B64</f>
         <v>1</v>
       </c>
-      <c r="D49" s="94" t="n">
+      <c r="D49" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G37)</f>
         <v>0</v>
       </c>
-      <c r="E49" s="94" t="n">
+      <c r="E49" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H37)</f>
         <v>0</v>
       </c>
@@ -5065,20 +5072,20 @@
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C50" s="94" t="n">
+      <c r="C50" s="90" t="n">
         <f aca="false">Auteur!B65</f>
         <v>2</v>
       </c>
-      <c r="D50" s="94" t="n">
+      <c r="D50" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G38)</f>
         <v>0</v>
       </c>
-      <c r="E50" s="94" t="n">
+      <c r="E50" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H38)</f>
         <v>0</v>
       </c>
@@ -5086,20 +5093,20 @@
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C51" s="94" t="n">
+      <c r="C51" s="90" t="n">
         <f aca="false">Auteur!B66</f>
         <v>3</v>
       </c>
-      <c r="D51" s="94" t="n">
+      <c r="D51" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G39)</f>
         <v>0</v>
       </c>
-      <c r="E51" s="94" t="n">
+      <c r="E51" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H39)</f>
         <v>0</v>
       </c>
@@ -5107,20 +5114,20 @@
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C52" s="94" t="n">
+      <c r="C52" s="90" t="n">
         <f aca="false">Auteur!B67</f>
         <v>4</v>
       </c>
-      <c r="D52" s="94" t="n">
+      <c r="D52" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G40)</f>
         <v>0</v>
       </c>
-      <c r="E52" s="94" t="n">
+      <c r="E52" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H40)</f>
         <v>0</v>
       </c>
@@ -5128,20 +5135,20 @@
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C53" s="94" t="n">
+      <c r="C53" s="90" t="n">
         <f aca="false">Auteur!B68</f>
         <v>5</v>
       </c>
-      <c r="D53" s="94" t="n">
+      <c r="D53" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G41)</f>
         <v>0</v>
       </c>
-      <c r="E53" s="94" t="n">
+      <c r="E53" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H41)</f>
         <v>0</v>
       </c>
@@ -5149,20 +5156,20 @@
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C54" s="94" t="n">
+      <c r="C54" s="90" t="n">
         <f aca="false">Auteur!B69</f>
         <v>6</v>
       </c>
-      <c r="D54" s="94" t="n">
+      <c r="D54" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G42)</f>
         <v>0</v>
       </c>
-      <c r="E54" s="94" t="n">
+      <c r="E54" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H42)</f>
         <v>0</v>
       </c>
@@ -5170,20 +5177,20 @@
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C55" s="94" t="n">
+      <c r="C55" s="90" t="n">
         <f aca="false">Auteur!B70</f>
         <v>7</v>
       </c>
-      <c r="D55" s="94" t="n">
+      <c r="D55" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G43)</f>
         <v>0</v>
       </c>
-      <c r="E55" s="94" t="n">
+      <c r="E55" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H43)</f>
         <v>0</v>
       </c>
@@ -5191,20 +5198,20 @@
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C56" s="94" t="n">
+      <c r="C56" s="90" t="n">
         <f aca="false">Auteur!B71</f>
         <v>8</v>
       </c>
-      <c r="D56" s="94" t="n">
+      <c r="D56" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G44)</f>
         <v>0</v>
       </c>
-      <c r="E56" s="94" t="n">
+      <c r="E56" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H44)</f>
         <v>0</v>
       </c>
@@ -5212,20 +5219,20 @@
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C57" s="94" t="n">
+      <c r="C57" s="90" t="n">
         <f aca="false">Auteur!B76</f>
         <v>1</v>
       </c>
-      <c r="D57" s="94" t="n">
+      <c r="D57" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G45)</f>
         <v>0</v>
       </c>
-      <c r="E57" s="94" t="n">
+      <c r="E57" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H45)</f>
         <v>0</v>
       </c>
@@ -5233,20 +5240,20 @@
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C58" s="94" t="n">
+      <c r="C58" s="90" t="n">
         <f aca="false">Auteur!B77</f>
         <v>2</v>
       </c>
-      <c r="D58" s="94" t="n">
+      <c r="D58" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G46)</f>
         <v>0</v>
       </c>
-      <c r="E58" s="94" t="n">
+      <c r="E58" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H46)</f>
         <v>0</v>
       </c>
@@ -5254,20 +5261,20 @@
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C59" s="94" t="n">
+      <c r="C59" s="90" t="n">
         <f aca="false">Auteur!B78</f>
         <v>3</v>
       </c>
-      <c r="D59" s="94" t="n">
+      <c r="D59" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G47)</f>
         <v>0</v>
       </c>
-      <c r="E59" s="94" t="n">
+      <c r="E59" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H47)</f>
         <v>0</v>
       </c>
@@ -5275,20 +5282,20 @@
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C60" s="94" t="n">
+      <c r="C60" s="90" t="n">
         <f aca="false">Auteur!B79</f>
         <v>4</v>
       </c>
-      <c r="D60" s="94" t="n">
+      <c r="D60" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G48)</f>
         <v>0</v>
       </c>
-      <c r="E60" s="94" t="n">
+      <c r="E60" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H48)</f>
         <v>0</v>
       </c>
@@ -5296,20 +5303,20 @@
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C61" s="94" t="n">
+      <c r="C61" s="90" t="n">
         <f aca="false">Auteur!B80</f>
         <v>5</v>
       </c>
-      <c r="D61" s="94" t="n">
+      <c r="D61" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G49)</f>
         <v>0</v>
       </c>
-      <c r="E61" s="94" t="n">
+      <c r="E61" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H49)</f>
         <v>0</v>
       </c>
@@ -5317,20 +5324,20 @@
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C62" s="94" t="n">
+      <c r="C62" s="90" t="n">
         <f aca="false">Auteur!B85</f>
         <v>1</v>
       </c>
-      <c r="D62" s="94" t="n">
+      <c r="D62" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G50)</f>
         <v>0</v>
       </c>
-      <c r="E62" s="94" t="n">
+      <c r="E62" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H50)</f>
         <v>0</v>
       </c>
@@ -5338,41 +5345,41 @@
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C63" s="94" t="n">
+      <c r="C63" s="90" t="n">
         <f aca="false">Auteur!B86</f>
         <v>2</v>
       </c>
-      <c r="D63" s="94" t="n">
+      <c r="D63" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G51)</f>
         <v>0</v>
       </c>
-      <c r="E63" s="94" t="n">
+      <c r="E63" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H51)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C64" s="94" t="n">
+      <c r="C64" s="90" t="n">
         <f aca="false">Auteur!B87</f>
         <v>3</v>
       </c>
-      <c r="D64" s="94" t="n">
+      <c r="D64" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G52)</f>
         <v>0</v>
       </c>
-      <c r="E64" s="94" t="n">
+      <c r="E64" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H52)</f>
         <v>0</v>
       </c>
@@ -5380,20 +5387,20 @@
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C65" s="94" t="n">
+      <c r="C65" s="90" t="n">
         <f aca="false">Auteur!B88</f>
         <v>4</v>
       </c>
-      <c r="D65" s="94" t="n">
+      <c r="D65" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G53)</f>
         <v>0</v>
       </c>
-      <c r="E65" s="94" t="n">
+      <c r="E65" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H53)</f>
         <v>0</v>
       </c>
@@ -5401,20 +5408,20 @@
     <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C66" s="94" t="n">
+      <c r="C66" s="90" t="n">
         <f aca="false">Auteur!B89</f>
         <v>5</v>
       </c>
-      <c r="D66" s="94" t="n">
+      <c r="D66" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G54)</f>
         <v>0</v>
       </c>
-      <c r="E66" s="94" t="n">
+      <c r="E66" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H54)</f>
         <v>0</v>
       </c>
@@ -5422,20 +5429,20 @@
     <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C67" s="94" t="n">
+      <c r="C67" s="90" t="n">
         <f aca="false">Auteur!B94</f>
         <v>1</v>
       </c>
-      <c r="D67" s="94" t="n">
+      <c r="D67" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G55)</f>
         <v>0</v>
       </c>
-      <c r="E67" s="94" t="n">
+      <c r="E67" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H55)</f>
         <v>0</v>
       </c>
@@ -5443,20 +5450,20 @@
     <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C68" s="94" t="n">
+      <c r="C68" s="90" t="n">
         <f aca="false">Auteur!B95</f>
         <v>2</v>
       </c>
-      <c r="D68" s="94" t="n">
+      <c r="D68" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G56)</f>
         <v>0</v>
       </c>
-      <c r="E68" s="94" t="n">
+      <c r="E68" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H56)</f>
         <v>0</v>
       </c>
@@ -5464,20 +5471,20 @@
     <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C69" s="94" t="n">
+      <c r="C69" s="90" t="n">
         <f aca="false">Auteur!B96</f>
         <v>3</v>
       </c>
-      <c r="D69" s="94" t="n">
+      <c r="D69" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G57)</f>
         <v>0</v>
       </c>
-      <c r="E69" s="94" t="n">
+      <c r="E69" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H57)</f>
         <v>0</v>
       </c>
@@ -5485,20 +5492,20 @@
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C70" s="94" t="n">
+      <c r="C70" s="90" t="n">
         <f aca="false">Auteur!B101</f>
         <v>1</v>
       </c>
-      <c r="D70" s="94" t="n">
+      <c r="D70" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G58)</f>
         <v>0</v>
       </c>
-      <c r="E70" s="94" t="n">
+      <c r="E70" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H58)</f>
         <v>0</v>
       </c>
@@ -5506,20 +5513,20 @@
     <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C71" s="94" t="n">
+      <c r="C71" s="90" t="n">
         <f aca="false">Auteur!B102</f>
         <v>2</v>
       </c>
-      <c r="D71" s="94" t="n">
+      <c r="D71" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G59)</f>
         <v>0</v>
       </c>
-      <c r="E71" s="94" t="n">
+      <c r="E71" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H59)</f>
         <v>0</v>
       </c>
@@ -5527,20 +5534,20 @@
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C72" s="94" t="n">
+      <c r="C72" s="90" t="n">
         <f aca="false">Auteur!B103</f>
         <v>3</v>
       </c>
-      <c r="D72" s="94" t="n">
+      <c r="D72" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G60)</f>
         <v>0</v>
       </c>
-      <c r="E72" s="94" t="n">
+      <c r="E72" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H60)</f>
         <v>0</v>
       </c>
@@ -5548,20 +5555,20 @@
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C73" s="94" t="n">
+      <c r="C73" s="90" t="n">
         <f aca="false">Auteur!B104</f>
         <v>4</v>
       </c>
-      <c r="D73" s="94" t="n">
+      <c r="D73" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G61)</f>
         <v>0</v>
       </c>
-      <c r="E73" s="94" t="n">
+      <c r="E73" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H61)</f>
         <v>0</v>
       </c>
@@ -5569,130 +5576,130 @@
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C74" s="94" t="n">
+      <c r="C74" s="90" t="n">
         <f aca="false">Auteur!B109</f>
         <v>1</v>
       </c>
-      <c r="D74" s="94" t="n">
+      <c r="D74" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G62)</f>
         <v>0</v>
       </c>
-      <c r="E74" s="94" t="n">
+      <c r="E74" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H62)</f>
         <v>0</v>
       </c>
-      <c r="IT74" s="94"/>
+      <c r="IT74" s="90"/>
     </row>
     <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C75" s="94" t="n">
+      <c r="C75" s="90" t="n">
         <f aca="false">Auteur!B110</f>
         <v>2</v>
       </c>
-      <c r="D75" s="94" t="n">
+      <c r="D75" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G63)</f>
         <v>0</v>
       </c>
-      <c r="E75" s="94" t="n">
+      <c r="E75" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H63)</f>
         <v>0</v>
       </c>
-      <c r="IT75" s="94"/>
+      <c r="IT75" s="90"/>
     </row>
     <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C76" s="94" t="n">
+      <c r="C76" s="90" t="n">
         <f aca="false">Auteur!B111</f>
         <v>3</v>
       </c>
-      <c r="D76" s="94" t="n">
+      <c r="D76" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G64)</f>
         <v>0</v>
       </c>
-      <c r="E76" s="94" t="n">
+      <c r="E76" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H64)</f>
         <v>0</v>
       </c>
-      <c r="IT76" s="94"/>
+      <c r="IT76" s="90"/>
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C77" s="94" t="n">
+      <c r="C77" s="90" t="n">
         <f aca="false">Auteur!B112</f>
         <v>4</v>
       </c>
-      <c r="D77" s="94" t="n">
+      <c r="D77" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G65)</f>
         <v>0</v>
       </c>
-      <c r="E77" s="94" t="n">
+      <c r="E77" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H65)</f>
         <v>0</v>
       </c>
-      <c r="IT77" s="94"/>
+      <c r="IT77" s="90"/>
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C78" s="94" t="n">
+      <c r="C78" s="90" t="n">
         <f aca="false">Auteur!B113</f>
         <v>5</v>
       </c>
-      <c r="D78" s="94" t="n">
+      <c r="D78" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G66)</f>
         <v>0</v>
       </c>
-      <c r="E78" s="94" t="n">
+      <c r="E78" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H66)</f>
         <v>0</v>
       </c>
-      <c r="IT78" s="94"/>
+      <c r="IT78" s="90"/>
     </row>
     <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C79" s="94" t="n">
+      <c r="C79" s="90" t="n">
         <f aca="false">Auteur!B118</f>
         <v>1</v>
       </c>
-      <c r="D79" s="94" t="n">
+      <c r="D79" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G67)</f>
         <v>0</v>
       </c>
-      <c r="E79" s="94" t="n">
+      <c r="E79" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H67)</f>
         <v>0</v>
       </c>
@@ -5700,20 +5707,20 @@
     <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C80" s="94" t="n">
+      <c r="C80" s="90" t="n">
         <f aca="false">Auteur!B119</f>
         <v>2</v>
       </c>
-      <c r="D80" s="94" t="n">
+      <c r="D80" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G68)</f>
         <v>0</v>
       </c>
-      <c r="E80" s="94" t="n">
+      <c r="E80" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H68)</f>
         <v>0</v>
       </c>
@@ -5721,20 +5728,20 @@
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C81" s="94" t="n">
+      <c r="C81" s="90" t="n">
         <f aca="false">Auteur!B120</f>
         <v>3</v>
       </c>
-      <c r="D81" s="94" t="n">
+      <c r="D81" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G69)</f>
         <v>0</v>
       </c>
-      <c r="E81" s="94" t="n">
+      <c r="E81" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H69)</f>
         <v>0</v>
       </c>
@@ -5742,20 +5749,20 @@
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C82" s="94" t="n">
+      <c r="C82" s="90" t="n">
         <f aca="false">Auteur!B121</f>
         <v>4</v>
       </c>
-      <c r="D82" s="94" t="n">
+      <c r="D82" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G70)</f>
         <v>0</v>
       </c>
-      <c r="E82" s="94" t="n">
+      <c r="E82" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H70)</f>
         <v>0</v>
       </c>
@@ -5763,20 +5770,20 @@
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C83" s="94" t="n">
+      <c r="C83" s="90" t="n">
         <f aca="false">Auteur!B122</f>
         <v>5</v>
       </c>
-      <c r="D83" s="94" t="n">
+      <c r="D83" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G71)</f>
         <v>0</v>
       </c>
-      <c r="E83" s="94" t="n">
+      <c r="E83" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H71)</f>
         <v>0</v>
       </c>
@@ -5784,465 +5791,457 @@
     <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C84" s="94" t="n">
+      <c r="C84" s="90" t="s">
+        <v>79</v>
+      </c>
+      <c r="D84" s="90" t="str">
+        <f aca="false">Auteur!C129</f>
+        <v>Saisir question thème 1 ici</v>
+      </c>
+      <c r="E84" s="90"/>
+    </row>
+    <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C85" s="90" t="n">
         <f aca="false">Auteur!B130</f>
         <v>1</v>
       </c>
-      <c r="D84" s="94" t="n">
+      <c r="D85" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G72)</f>
         <v>0</v>
       </c>
-      <c r="E84" s="94" t="n">
+      <c r="E85" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H72)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B85" s="2" t="n">
+    <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B86" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C85" s="94" t="n">
+      <c r="C86" s="90" t="n">
         <f aca="false">Auteur!B131</f>
         <v>2</v>
       </c>
-      <c r="D85" s="94" t="n">
+      <c r="D86" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G73)</f>
         <v>0</v>
       </c>
-      <c r="E85" s="94" t="n">
+      <c r="E86" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H73)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B86" s="2" t="n">
+    <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B87" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C86" s="94" t="n">
+      <c r="C87" s="90" t="n">
         <f aca="false">Auteur!B132</f>
         <v>3</v>
       </c>
-      <c r="D86" s="94" t="n">
+      <c r="D87" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G74)</f>
         <v>0</v>
       </c>
-      <c r="E86" s="94" t="n">
+      <c r="E87" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H74)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B87" s="2" t="n">
+    <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B88" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C87" s="94" t="n">
+      <c r="C88" s="90" t="n">
         <f aca="false">Auteur!B133</f>
         <v>4</v>
       </c>
-      <c r="D87" s="94" t="n">
+      <c r="D88" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G75)</f>
         <v>0</v>
       </c>
-      <c r="E87" s="94" t="n">
+      <c r="E88" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H75)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B88" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="C88" s="94" t="n">
-        <v>5</v>
-      </c>
-      <c r="D88" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!G76)</f>
-        <v>0</v>
-      </c>
-      <c r="E88" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!H76)</f>
         <v>0</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C89" s="94" t="n">
-        <v>6</v>
-      </c>
-      <c r="D89" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!G77)</f>
-        <v>0</v>
-      </c>
-      <c r="E89" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!H77)</f>
-        <v>0</v>
-      </c>
+      <c r="C89" s="90" t="s">
+        <v>80</v>
+      </c>
+      <c r="D89" s="90" t="str">
+        <f aca="false">Auteur!C140</f>
+        <v>Saisir question thème 2 ici</v>
+      </c>
+      <c r="E89" s="90"/>
     </row>
     <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C90" s="94" t="n">
-        <v>7</v>
-      </c>
-      <c r="D90" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!G78)</f>
-        <v>0</v>
-      </c>
-      <c r="E90" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!H78)</f>
+      <c r="C90" s="90" t="n">
+        <v>5</v>
+      </c>
+      <c r="D90" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!G76)</f>
+        <v>0</v>
+      </c>
+      <c r="E90" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!H76)</f>
         <v>0</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C91" s="94" t="n">
-        <v>8</v>
-      </c>
-      <c r="D91" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!G79)</f>
-        <v>0</v>
-      </c>
-      <c r="E91" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!H79)</f>
+      <c r="C91" s="90" t="n">
+        <v>6</v>
+      </c>
+      <c r="D91" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!G77)</f>
+        <v>0</v>
+      </c>
+      <c r="E91" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!H77)</f>
         <v>0</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B92" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="C92" s="94" t="n">
-        <v>1</v>
-      </c>
-      <c r="D92" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!G80)</f>
-        <v>0</v>
-      </c>
-      <c r="E92" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!H80)</f>
-        <v>0</v>
-      </c>
-      <c r="IT92" s="94"/>
+        <v>13</v>
+      </c>
+      <c r="C92" s="90" t="n">
+        <v>7</v>
+      </c>
+      <c r="D92" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!G78)</f>
+        <v>0</v>
+      </c>
+      <c r="E92" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!H78)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B93" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="C93" s="94" t="n">
-        <v>2</v>
-      </c>
-      <c r="D93" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!G81)</f>
-        <v>0</v>
-      </c>
-      <c r="E93" s="94" t="n">
-        <f aca="true">INDIRECT(Adresses!H81)</f>
-        <v>0</v>
-      </c>
-      <c r="IT93" s="94"/>
+        <v>13</v>
+      </c>
+      <c r="C93" s="90" t="n">
+        <v>8</v>
+      </c>
+      <c r="D93" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!G79)</f>
+        <v>0</v>
+      </c>
+      <c r="E93" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!H79)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C94" s="94" t="n">
+      <c r="C94" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!G80)</f>
+        <v>0</v>
+      </c>
+      <c r="E94" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!H80)</f>
+        <v>0</v>
+      </c>
+      <c r="IT94" s="90"/>
+    </row>
+    <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C95" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D95" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!G81)</f>
+        <v>0</v>
+      </c>
+      <c r="E95" s="90" t="n">
+        <f aca="true">INDIRECT(Adresses!H81)</f>
+        <v>0</v>
+      </c>
+      <c r="IT95" s="90"/>
+    </row>
+    <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C96" s="90" t="n">
         <f aca="false">Auteur!B155</f>
         <v>3</v>
       </c>
-      <c r="D94" s="94" t="n">
+      <c r="D96" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G82)</f>
         <v>0</v>
       </c>
-      <c r="E94" s="94" t="n">
+      <c r="E96" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H82)</f>
         <v>0</v>
       </c>
-      <c r="IT94" s="94"/>
-    </row>
-    <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B95" s="2" t="n">
+      <c r="IT96" s="90"/>
+    </row>
+    <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B97" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C95" s="94" t="n">
+      <c r="C97" s="90" t="n">
         <f aca="false">Auteur!B156</f>
         <v>4</v>
       </c>
-      <c r="D95" s="94" t="n">
+      <c r="D97" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G83)</f>
         <v>0</v>
       </c>
-      <c r="E95" s="94" t="n">
+      <c r="E97" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H83)</f>
         <v>0</v>
       </c>
-      <c r="IT95" s="94"/>
-    </row>
-    <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B96" s="2" t="n">
+      <c r="IT97" s="90"/>
+    </row>
+    <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B98" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C96" s="94" t="n">
+      <c r="C98" s="90" t="n">
         <f aca="false">Auteur!B157</f>
         <v>5</v>
       </c>
-      <c r="D96" s="94" t="n">
+      <c r="D98" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G84)</f>
         <v>0</v>
       </c>
-      <c r="E96" s="94" t="n">
+      <c r="E98" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H84)</f>
         <v>0</v>
       </c>
-      <c r="IT96" s="95"/>
-    </row>
-    <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B97" s="2" t="n">
+      <c r="IT98" s="91"/>
+    </row>
+    <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B99" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C97" s="94" t="n">
+      <c r="C99" s="90" t="n">
         <f aca="false">Auteur!B158</f>
         <v>6</v>
       </c>
-      <c r="D97" s="94" t="n">
+      <c r="D99" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G85)</f>
         <v>0</v>
       </c>
-      <c r="E97" s="94" t="n">
+      <c r="E99" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H85)</f>
         <v>0</v>
       </c>
-      <c r="IT97" s="95"/>
-    </row>
-    <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B98" s="2" t="n">
+      <c r="IT99" s="91"/>
+    </row>
+    <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B100" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C98" s="94" t="n">
+      <c r="C100" s="90" t="n">
         <f aca="false">Auteur!B159</f>
         <v>7</v>
       </c>
-      <c r="D98" s="94" t="n">
+      <c r="D100" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G86)</f>
         <v>0</v>
       </c>
-      <c r="E98" s="94" t="n">
+      <c r="E100" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H86)</f>
         <v>0</v>
       </c>
-      <c r="IT98" s="95"/>
-    </row>
-    <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B99" s="2" t="n">
+      <c r="IT100" s="91"/>
+    </row>
+    <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B101" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C99" s="94" t="n">
+      <c r="C101" s="90" t="n">
         <f aca="false">Auteur!B160</f>
         <v>8</v>
       </c>
-      <c r="D99" s="94" t="n">
+      <c r="D101" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G87)</f>
         <v>0</v>
       </c>
-      <c r="E99" s="94" t="n">
+      <c r="E101" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H87)</f>
         <v>0</v>
       </c>
-      <c r="IT99" s="95"/>
-    </row>
-    <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B100" s="2" t="n">
+      <c r="IT101" s="91"/>
+    </row>
+    <row r="102" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B102" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C100" s="94" t="n">
+      <c r="C102" s="90" t="n">
         <f aca="false">Auteur!B161</f>
         <v>9</v>
       </c>
-      <c r="D100" s="94" t="n">
+      <c r="D102" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G88)</f>
         <v>0</v>
       </c>
-      <c r="E100" s="94" t="n">
+      <c r="E102" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H88)</f>
         <v>0</v>
       </c>
-      <c r="IT100" s="95"/>
-    </row>
-    <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B101" s="2" t="n">
+      <c r="IT102" s="91"/>
+    </row>
+    <row r="103" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B103" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C101" s="94" t="n">
+      <c r="C103" s="90" t="n">
         <f aca="false">Auteur!B162</f>
         <v>10</v>
       </c>
-      <c r="D101" s="94" t="n">
+      <c r="D103" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G89)</f>
         <v>0</v>
       </c>
-      <c r="E101" s="94" t="n">
+      <c r="E103" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H89)</f>
         <v>0</v>
       </c>
-      <c r="IT101" s="95"/>
-    </row>
-    <row r="102" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B102" s="2" t="n">
+      <c r="IT103" s="91"/>
+    </row>
+    <row r="104" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B104" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C102" s="94" t="n">
+      <c r="C104" s="90" t="n">
         <f aca="false">Auteur!B167</f>
         <v>1</v>
       </c>
-      <c r="D102" s="94" t="n">
+      <c r="D104" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!G90)</f>
         <v>0</v>
       </c>
-      <c r="E102" s="94" t="n">
+      <c r="E104" s="90" t="n">
         <f aca="true">INDIRECT(Adresses!H90)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B103" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C103" s="94" t="n">
-        <f aca="false">C102+1</f>
-        <v>2</v>
-      </c>
-      <c r="D103" s="94" t="n">
-        <f aca="false">$D$102</f>
-        <v>0</v>
-      </c>
-      <c r="E103" s="94" t="n">
-        <f aca="false">E102</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
-      </c>
-      <c r="B104" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C104" s="94" t="n">
-        <f aca="false">C103+1</f>
-        <v>3</v>
-      </c>
-      <c r="D104" s="94" t="n">
-        <f aca="false">$D$102</f>
-        <v>0</v>
-      </c>
-      <c r="E104" s="94" t="n">
-        <f aca="false">E103</f>
         <v>0</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C105" s="94" t="n">
+      <c r="C105" s="90" t="n">
         <f aca="false">C104+1</f>
-        <v>4</v>
-      </c>
-      <c r="D105" s="94" t="n">
-        <f aca="false">$D$102</f>
-        <v>0</v>
-      </c>
-      <c r="E105" s="94" t="n">
+        <v>2</v>
+      </c>
+      <c r="D105" s="90" t="n">
+        <f aca="false">$D$104</f>
+        <v>0</v>
+      </c>
+      <c r="E105" s="90" t="n">
         <f aca="false">E104</f>
         <v>0</v>
       </c>
@@ -6250,20 +6249,20 @@
     <row r="106" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C106" s="94" t="n">
+      <c r="C106" s="90" t="n">
         <f aca="false">C105+1</f>
-        <v>5</v>
-      </c>
-      <c r="D106" s="94" t="n">
-        <f aca="false">$D$102</f>
-        <v>0</v>
-      </c>
-      <c r="E106" s="94" t="n">
+        <v>3</v>
+      </c>
+      <c r="D106" s="90" t="n">
+        <f aca="false">$D$104</f>
+        <v>0</v>
+      </c>
+      <c r="E106" s="90" t="n">
         <f aca="false">E105</f>
         <v>0</v>
       </c>
@@ -6271,20 +6270,20 @@
     <row r="107" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C107" s="94" t="n">
+      <c r="C107" s="90" t="n">
         <f aca="false">C106+1</f>
-        <v>6</v>
-      </c>
-      <c r="D107" s="94" t="n">
-        <f aca="false">$D$102</f>
-        <v>0</v>
-      </c>
-      <c r="E107" s="94" t="n">
+        <v>4</v>
+      </c>
+      <c r="D107" s="90" t="n">
+        <f aca="false">$D$104</f>
+        <v>0</v>
+      </c>
+      <c r="E107" s="90" t="n">
         <f aca="false">E106</f>
         <v>0</v>
       </c>
@@ -6292,20 +6291,20 @@
     <row r="108" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C108" s="94" t="n">
+      <c r="C108" s="90" t="n">
         <f aca="false">C107+1</f>
-        <v>7</v>
-      </c>
-      <c r="D108" s="94" t="n">
-        <f aca="false">$D$102</f>
-        <v>0</v>
-      </c>
-      <c r="E108" s="94" t="n">
+        <v>5</v>
+      </c>
+      <c r="D108" s="90" t="n">
+        <f aca="false">$D$104</f>
+        <v>0</v>
+      </c>
+      <c r="E108" s="90" t="n">
         <f aca="false">E107</f>
         <v>0</v>
       </c>
@@ -6313,21 +6312,63 @@
     <row r="109" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="n">
         <f aca="false">Auteur!$D$2</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C109" s="94" t="n">
+      <c r="C109" s="90" t="n">
         <f aca="false">C108+1</f>
+        <v>6</v>
+      </c>
+      <c r="D109" s="90" t="n">
+        <f aca="false">$D$104</f>
+        <v>0</v>
+      </c>
+      <c r="E109" s="90" t="n">
+        <f aca="false">E108</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C110" s="90" t="n">
+        <f aca="false">C109+1</f>
+        <v>7</v>
+      </c>
+      <c r="D110" s="90" t="n">
+        <f aca="false">$D$104</f>
+        <v>0</v>
+      </c>
+      <c r="E110" s="90" t="n">
+        <f aca="false">E109</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C111" s="90" t="n">
+        <f aca="false">C110+1</f>
         <v>8</v>
       </c>
-      <c r="D109" s="94" t="n">
-        <f aca="false">$D$102</f>
-        <v>0</v>
-      </c>
-      <c r="E109" s="94" t="n">
-        <f aca="false">E108</f>
+      <c r="D111" s="90" t="n">
+        <f aca="false">$D$104</f>
+        <v>0</v>
+      </c>
+      <c r="E111" s="90" t="n">
+        <f aca="false">E110</f>
         <v>0</v>
       </c>
     </row>
@@ -6357,77 +6398,77 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="96" t="s">
+      <c r="A2" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="97" t="n">
+      <c r="B2" s="92"/>
+      <c r="C2" s="93" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="97"/>
+      <c r="D2" s="93"/>
       <c r="G2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="98"/>
-      <c r="C3" s="99" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" s="99"/>
+      <c r="B3" s="94"/>
+      <c r="C3" s="95" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" s="95"/>
       <c r="G3" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="98" t="s">
+      <c r="A4" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="98"/>
-      <c r="C4" s="99" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="99"/>
+      <c r="B4" s="94"/>
+      <c r="C4" s="95" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="95"/>
       <c r="G4" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="98" t="s">
+      <c r="A5" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="98"/>
-      <c r="C5" s="99" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" s="99"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="95" t="s">
+        <v>84</v>
+      </c>
+      <c r="D5" s="95"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="98" t="s">
-        <v>81</v>
-      </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="99"/>
-      <c r="D6" s="99"/>
+      <c r="A6" s="94" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="94"/>
+      <c r="C6" s="95"/>
+      <c r="D6" s="95"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="98" t="s">
-        <v>82</v>
-      </c>
-      <c r="B7" s="98"/>
-      <c r="C7" s="99"/>
-      <c r="D7" s="99"/>
+      <c r="A7" s="94" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="94"/>
+      <c r="C7" s="95"/>
+      <c r="D7" s="95"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="100" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="100"/>
-      <c r="C8" s="101"/>
-      <c r="D8" s="101"/>
+      <c r="A8" s="96" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="96"/>
+      <c r="C8" s="97"/>
+      <c r="D8" s="97"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10"/>
@@ -6436,165 +6477,165 @@
       <c r="D9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="102" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="102"/>
-      <c r="C10" s="102"/>
-      <c r="D10" s="102"/>
+      <c r="A10" s="98" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="98"/>
+      <c r="C10" s="98"/>
+      <c r="D10" s="98"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="103"/>
-      <c r="B11" s="103"/>
-      <c r="C11" s="103"/>
-      <c r="D11" s="103"/>
+      <c r="A11" s="99"/>
+      <c r="B11" s="99"/>
+      <c r="C11" s="99"/>
+      <c r="D11" s="99"/>
     </row>
     <row r="12" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="104" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="104"/>
-      <c r="C12" s="104" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="105"/>
+      <c r="A12" s="100" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="100"/>
+      <c r="C12" s="100" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="101"/>
     </row>
     <row r="13" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="106" t="s">
+      <c r="A13" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="106"/>
-      <c r="C13" s="107" t="s">
-        <v>86</v>
-      </c>
-      <c r="D13" s="108" t="s">
-        <v>87</v>
+      <c r="B13" s="102"/>
+      <c r="C13" s="103" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="104" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="109" t="s">
+      <c r="A14" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="109"/>
-      <c r="C14" s="109"/>
-      <c r="D14" s="109"/>
+      <c r="B14" s="105"/>
+      <c r="C14" s="105"/>
+      <c r="D14" s="105"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="109"/>
-      <c r="B15" s="109"/>
-      <c r="C15" s="109"/>
-      <c r="D15" s="109"/>
+      <c r="A15" s="105"/>
+      <c r="B15" s="105"/>
+      <c r="C15" s="105"/>
+      <c r="D15" s="105"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="109"/>
-      <c r="B16" s="109"/>
-      <c r="C16" s="109"/>
-      <c r="D16" s="109"/>
+      <c r="A16" s="105"/>
+      <c r="B16" s="105"/>
+      <c r="C16" s="105"/>
+      <c r="D16" s="105"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="110" t="n">
+      <c r="A17" s="106" t="n">
         <v>1</v>
       </c>
-      <c r="B17" s="111" t="n">
+      <c r="B17" s="107" t="n">
         <f aca="false">'Vers BD'!D22</f>
         <v>0</v>
       </c>
-      <c r="C17" s="111"/>
-      <c r="D17" s="112" t="n">
+      <c r="C17" s="107"/>
+      <c r="D17" s="108" t="n">
         <f aca="false">'Vers BD'!E22</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="110" t="n">
+      <c r="A18" s="106" t="n">
         <v>2</v>
       </c>
-      <c r="B18" s="111" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="111"/>
-      <c r="D18" s="112" t="s">
-        <v>89</v>
+      <c r="B18" s="107" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" s="107"/>
+      <c r="D18" s="108" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="110" t="n">
+      <c r="A19" s="106" t="n">
         <v>3</v>
       </c>
-      <c r="B19" s="111" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="111"/>
-      <c r="D19" s="112" t="s">
-        <v>91</v>
+      <c r="B19" s="107" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="107"/>
+      <c r="D19" s="108" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="110" t="n">
+      <c r="A20" s="106" t="n">
         <v>4</v>
       </c>
-      <c r="B20" s="111" t="s">
-        <v>92</v>
-      </c>
-      <c r="C20" s="111"/>
-      <c r="D20" s="112" t="s">
-        <v>93</v>
+      <c r="B20" s="107" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" s="107"/>
+      <c r="D20" s="108" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="109" t="s">
+      <c r="A21" s="105" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="109"/>
-      <c r="C21" s="109"/>
-      <c r="D21" s="109"/>
+      <c r="B21" s="105"/>
+      <c r="C21" s="105"/>
+      <c r="D21" s="105"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="110" t="n">
+      <c r="A22" s="106" t="n">
         <v>1</v>
       </c>
-      <c r="B22" s="111" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" s="111"/>
-      <c r="D22" s="112" t="s">
-        <v>95</v>
+      <c r="B22" s="107" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="107"/>
+      <c r="D22" s="108" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="110" t="n">
+      <c r="A23" s="106" t="n">
         <v>2</v>
       </c>
-      <c r="B23" s="111" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="111"/>
-      <c r="D23" s="112" t="s">
-        <v>97</v>
+      <c r="B23" s="107" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="107"/>
+      <c r="D23" s="108" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="110" t="n">
+      <c r="A24" s="106" t="n">
         <v>3</v>
       </c>
-      <c r="B24" s="111" t="s">
-        <v>98</v>
-      </c>
-      <c r="C24" s="111"/>
-      <c r="D24" s="112" t="s">
-        <v>99</v>
+      <c r="B24" s="107" t="s">
+        <v>102</v>
+      </c>
+      <c r="C24" s="107"/>
+      <c r="D24" s="108" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="110" t="n">
+      <c r="A25" s="106" t="n">
         <v>4</v>
       </c>
-      <c r="B25" s="111" t="s">
-        <v>100</v>
-      </c>
-      <c r="C25" s="111"/>
-      <c r="D25" s="112" t="s">
-        <v>101</v>
+      <c r="B25" s="107" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" s="107"/>
+      <c r="D25" s="108" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6604,97 +6645,97 @@
       <c r="D26" s="28"/>
     </row>
     <row r="27" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="102" t="s">
-        <v>102</v>
-      </c>
-      <c r="B27" s="102"/>
-      <c r="C27" s="102"/>
-      <c r="D27" s="102"/>
+      <c r="A27" s="98" t="s">
+        <v>106</v>
+      </c>
+      <c r="B27" s="98"/>
+      <c r="C27" s="98"/>
+      <c r="D27" s="98"/>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="103"/>
-      <c r="B28" s="103"/>
-      <c r="C28" s="103"/>
-      <c r="D28" s="103"/>
+      <c r="A28" s="99"/>
+      <c r="B28" s="99"/>
+      <c r="C28" s="99"/>
+      <c r="D28" s="99"/>
     </row>
     <row r="29" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="104" t="s">
-        <v>103</v>
-      </c>
-      <c r="B29" s="104"/>
-      <c r="C29" s="113" t="s">
-        <v>71</v>
-      </c>
-      <c r="D29" s="114" t="s">
-        <v>104</v>
+      <c r="A29" s="100" t="s">
+        <v>107</v>
+      </c>
+      <c r="B29" s="100"/>
+      <c r="C29" s="109" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="110" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="115" t="s">
-        <v>105</v>
-      </c>
-      <c r="B30" s="115"/>
-      <c r="C30" s="113"/>
-      <c r="D30" s="114"/>
+      <c r="A30" s="111" t="s">
+        <v>109</v>
+      </c>
+      <c r="B30" s="111"/>
+      <c r="C30" s="109"/>
+      <c r="D30" s="110"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="110" t="n">
+      <c r="A31" s="106" t="n">
         <v>1</v>
       </c>
-      <c r="B31" s="111" t="s">
-        <v>106</v>
-      </c>
-      <c r="C31" s="111"/>
-      <c r="D31" s="112" t="s">
-        <v>107</v>
+      <c r="B31" s="107" t="s">
+        <v>110</v>
+      </c>
+      <c r="C31" s="107"/>
+      <c r="D31" s="108" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="110" t="n">
+      <c r="A32" s="106" t="n">
         <v>2</v>
       </c>
-      <c r="B32" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="C32" s="111"/>
-      <c r="D32" s="112" t="s">
-        <v>109</v>
+      <c r="B32" s="107" t="s">
+        <v>112</v>
+      </c>
+      <c r="C32" s="107"/>
+      <c r="D32" s="108" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="110" t="n">
+      <c r="A33" s="106" t="n">
         <v>3</v>
       </c>
-      <c r="B33" s="111" t="s">
-        <v>110</v>
-      </c>
-      <c r="C33" s="111"/>
-      <c r="D33" s="112" t="s">
-        <v>111</v>
+      <c r="B33" s="107" t="s">
+        <v>114</v>
+      </c>
+      <c r="C33" s="107"/>
+      <c r="D33" s="108" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="110" t="n">
+      <c r="A34" s="106" t="n">
         <v>4</v>
       </c>
-      <c r="B34" s="111" t="s">
-        <v>112</v>
-      </c>
-      <c r="C34" s="111"/>
-      <c r="D34" s="112" t="s">
-        <v>113</v>
+      <c r="B34" s="107" t="s">
+        <v>116</v>
+      </c>
+      <c r="C34" s="107"/>
+      <c r="D34" s="108" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="110" t="n">
+      <c r="A35" s="106" t="n">
         <v>5</v>
       </c>
-      <c r="B35" s="111" t="s">
-        <v>114</v>
-      </c>
-      <c r="C35" s="111"/>
-      <c r="D35" s="112" t="s">
-        <v>115</v>
+      <c r="B35" s="107" t="s">
+        <v>118</v>
+      </c>
+      <c r="C35" s="107"/>
+      <c r="D35" s="108" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6704,92 +6745,92 @@
       <c r="D36" s="34"/>
     </row>
     <row r="37" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="104" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="104"/>
-      <c r="C37" s="113" t="s">
-        <v>71</v>
-      </c>
-      <c r="D37" s="114" t="s">
-        <v>117</v>
+      <c r="A37" s="100" t="s">
+        <v>120</v>
+      </c>
+      <c r="B37" s="100"/>
+      <c r="C37" s="109" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" s="110" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="115" t="s">
-        <v>105</v>
-      </c>
-      <c r="B38" s="115"/>
-      <c r="C38" s="113"/>
-      <c r="D38" s="114"/>
+      <c r="A38" s="111" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" s="111"/>
+      <c r="C38" s="109"/>
+      <c r="D38" s="110"/>
     </row>
     <row r="39" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="110" t="n">
+      <c r="A39" s="106" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="111" t="s">
-        <v>118</v>
-      </c>
-      <c r="C39" s="111"/>
-      <c r="D39" s="112" t="s">
-        <v>119</v>
+      <c r="B39" s="107" t="s">
+        <v>122</v>
+      </c>
+      <c r="C39" s="107"/>
+      <c r="D39" s="108" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="110" t="n">
+      <c r="A40" s="106" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="111" t="s">
-        <v>120</v>
-      </c>
-      <c r="C40" s="111"/>
-      <c r="D40" s="112" t="s">
-        <v>121</v>
+      <c r="B40" s="107" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" s="107"/>
+      <c r="D40" s="108" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="110" t="n">
+      <c r="A41" s="106" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="111" t="s">
-        <v>122</v>
-      </c>
-      <c r="C41" s="111"/>
-      <c r="D41" s="112" t="s">
-        <v>123</v>
+      <c r="B41" s="107" t="s">
+        <v>126</v>
+      </c>
+      <c r="C41" s="107"/>
+      <c r="D41" s="108" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="110" t="n">
+      <c r="A42" s="106" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="111" t="s">
-        <v>124</v>
-      </c>
-      <c r="C42" s="111"/>
-      <c r="D42" s="112" t="s">
-        <v>125</v>
+      <c r="B42" s="107" t="s">
+        <v>128</v>
+      </c>
+      <c r="C42" s="107"/>
+      <c r="D42" s="108" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="111" t="n">
+      <c r="A43" s="107" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="116" t="s">
-        <v>126</v>
-      </c>
-      <c r="C43" s="116"/>
-      <c r="D43" s="117" t="s">
-        <v>127</v>
+      <c r="B43" s="112" t="s">
+        <v>130</v>
+      </c>
+      <c r="C43" s="112"/>
+      <c r="D43" s="113" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="77.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="111"/>
-      <c r="B44" s="110" t="s">
-        <v>128</v>
-      </c>
-      <c r="C44" s="110"/>
-      <c r="D44" s="117"/>
+      <c r="A44" s="107"/>
+      <c r="B44" s="106" t="s">
+        <v>132</v>
+      </c>
+      <c r="C44" s="106"/>
+      <c r="D44" s="113"/>
     </row>
   </sheetData>
   <mergeCells count="54">
@@ -6877,74 +6918,74 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="118" t="s">
-        <v>129</v>
+      <c r="A1" s="114" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="119" t="s">
-        <v>136</v>
-      </c>
-      <c r="B8" s="120" t="s">
-        <v>137</v>
-      </c>
-      <c r="C8" s="120" t="s">
-        <v>138</v>
-      </c>
-      <c r="D8" s="120" t="s">
-        <v>139</v>
-      </c>
-      <c r="E8" s="120" t="s">
+      <c r="A8" s="115" t="s">
         <v>140</v>
       </c>
-      <c r="F8" s="120" t="s">
+      <c r="B8" s="116" t="s">
         <v>141</v>
       </c>
-      <c r="G8" s="120" t="s">
+      <c r="C8" s="116" t="s">
         <v>142</v>
       </c>
-      <c r="H8" s="120" t="s">
+      <c r="D8" s="116" t="s">
         <v>143</v>
+      </c>
+      <c r="E8" s="116" t="s">
+        <v>144</v>
+      </c>
+      <c r="F8" s="116" t="s">
+        <v>145</v>
+      </c>
+      <c r="G8" s="116" t="s">
+        <v>146</v>
+      </c>
+      <c r="H8" s="116" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6966,7 +7007,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D9</f>
         <v>Auteur!D11</v>
       </c>
-      <c r="F9" s="118" t="n">
+      <c r="F9" s="114" t="n">
         <v>14</v>
       </c>
       <c r="G9" s="2" t="str">
@@ -7116,7 +7157,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D17</f>
         <v>Auteur!D25</v>
       </c>
-      <c r="F17" s="118" t="n">
+      <c r="F17" s="114" t="n">
         <v>27</v>
       </c>
       <c r="G17" s="2" t="str">
@@ -7216,7 +7257,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D22</f>
         <v>Auteur!D34</v>
       </c>
-      <c r="F22" s="118" t="n">
+      <c r="F22" s="114" t="n">
         <v>36</v>
       </c>
       <c r="G22" s="2" t="str">
@@ -7316,7 +7357,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D27</f>
         <v>Auteur!D43</v>
       </c>
-      <c r="F27" s="118" t="n">
+      <c r="F27" s="114" t="n">
         <v>45</v>
       </c>
       <c r="G27" s="2" t="str">
@@ -7416,7 +7457,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D32</f>
         <v>Auteur!D52</v>
       </c>
-      <c r="F32" s="118" t="n">
+      <c r="F32" s="114" t="n">
         <v>54</v>
       </c>
       <c r="G32" s="2" t="str">
@@ -7516,7 +7557,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D37</f>
         <v>Auteur!D61</v>
       </c>
-      <c r="F37" s="118" t="n">
+      <c r="F37" s="114" t="n">
         <v>64</v>
       </c>
       <c r="G37" s="2" t="str">
@@ -7583,7 +7624,7 @@
       <c r="A41" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F41" s="118" t="n">
+      <c r="F41" s="114" t="n">
         <v>68</v>
       </c>
       <c r="G41" s="2" t="str">
@@ -7666,7 +7707,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D45</f>
         <v>Auteur!D74</v>
       </c>
-      <c r="F45" s="118" t="n">
+      <c r="F45" s="114" t="n">
         <v>76</v>
       </c>
       <c r="G45" s="2" t="str">
@@ -7766,7 +7807,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D50</f>
         <v>Auteur!D83</v>
       </c>
-      <c r="F50" s="118" t="n">
+      <c r="F50" s="114" t="n">
         <v>85</v>
       </c>
       <c r="G50" s="2" t="str">
@@ -7866,7 +7907,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D55</f>
         <v>Auteur!D92</v>
       </c>
-      <c r="F55" s="118" t="n">
+      <c r="F55" s="114" t="n">
         <v>94</v>
       </c>
       <c r="G55" s="2" t="str">
@@ -7932,7 +7973,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D58</f>
         <v>Auteur!D99</v>
       </c>
-      <c r="F58" s="118" t="n">
+      <c r="F58" s="114" t="n">
         <v>101</v>
       </c>
       <c r="G58" s="2" t="str">
@@ -8015,7 +8056,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D62</f>
         <v>Auteur!D107</v>
       </c>
-      <c r="F62" s="118" t="n">
+      <c r="F62" s="114" t="n">
         <v>109</v>
       </c>
       <c r="G62" s="2" t="str">
@@ -8118,7 +8159,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D67</f>
         <v>Auteur!D116</v>
       </c>
-      <c r="F67" s="118" t="n">
+      <c r="F67" s="114" t="n">
         <v>118</v>
       </c>
       <c r="G67" s="2" t="str">
@@ -8200,41 +8241,41 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="121" t="n">
+      <c r="A72" s="117" t="n">
         <v>13</v>
       </c>
-      <c r="B72" s="122" t="n">
+      <c r="B72" s="118" t="n">
         <v>124</v>
       </c>
-      <c r="C72" s="122" t="str">
+      <c r="C72" s="118" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;B72</f>
         <v>Auteur!D124</v>
       </c>
-      <c r="D72" s="122" t="n">
+      <c r="D72" s="118" t="n">
         <v>125</v>
       </c>
-      <c r="E72" s="122" t="str">
+      <c r="E72" s="118" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D72</f>
         <v>Auteur!D125</v>
       </c>
-      <c r="F72" s="123" t="n">
+      <c r="F72" s="119" t="n">
         <v>130</v>
       </c>
-      <c r="G72" s="122" t="str">
+      <c r="G72" s="118" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F72</f>
         <v>Auteur!C130</v>
       </c>
-      <c r="H72" s="124" t="str">
+      <c r="H72" s="120" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F72</f>
         <v>Auteur!D130</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="125" t="n">
+      <c r="A73" s="121" t="n">
         <f aca="false">A69+1</f>
         <v>13</v>
       </c>
-      <c r="F73" s="126" t="n">
+      <c r="F73" s="122" t="n">
         <f aca="false">F72+1</f>
         <v>131</v>
       </c>
@@ -8242,16 +8283,16 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F73</f>
         <v>Auteur!C131</v>
       </c>
-      <c r="H73" s="127" t="str">
+      <c r="H73" s="123" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F73</f>
         <v>Auteur!D131</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="125" t="n">
+      <c r="A74" s="121" t="n">
         <v>13</v>
       </c>
-      <c r="F74" s="126" t="n">
+      <c r="F74" s="122" t="n">
         <f aca="false">F73+1</f>
         <v>132</v>
       </c>
@@ -8259,16 +8300,16 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F74</f>
         <v>Auteur!C132</v>
       </c>
-      <c r="H74" s="127" t="str">
+      <c r="H74" s="123" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F74</f>
         <v>Auteur!D132</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="125" t="n">
+      <c r="A75" s="121" t="n">
         <v>13</v>
       </c>
-      <c r="F75" s="126" t="n">
+      <c r="F75" s="122" t="n">
         <f aca="false">F74+1</f>
         <v>133</v>
       </c>
@@ -8276,75 +8317,75 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F75</f>
         <v>Auteur!C133</v>
       </c>
-      <c r="H75" s="127" t="str">
+      <c r="H75" s="123" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F75</f>
         <v>Auteur!D133</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="125" t="n">
+      <c r="A76" s="121" t="n">
         <v>13</v>
       </c>
-      <c r="F76" s="126" t="n">
+      <c r="F76" s="122" t="n">
         <v>141</v>
       </c>
       <c r="G76" s="2" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F76</f>
         <v>Auteur!C141</v>
       </c>
-      <c r="H76" s="127" t="str">
+      <c r="H76" s="123" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F76</f>
         <v>Auteur!D141</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="125" t="n">
+      <c r="A77" s="121" t="n">
         <v>13</v>
       </c>
-      <c r="F77" s="126" t="n">
+      <c r="F77" s="122" t="n">
         <v>142</v>
       </c>
       <c r="G77" s="2" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F77</f>
         <v>Auteur!C142</v>
       </c>
-      <c r="H77" s="127" t="str">
+      <c r="H77" s="123" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F77</f>
         <v>Auteur!D142</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="125" t="n">
+      <c r="A78" s="121" t="n">
         <v>13</v>
       </c>
-      <c r="F78" s="126" t="n">
+      <c r="F78" s="122" t="n">
         <v>143</v>
       </c>
       <c r="G78" s="2" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F78</f>
         <v>Auteur!C143</v>
       </c>
-      <c r="H78" s="127" t="str">
+      <c r="H78" s="123" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F78</f>
         <v>Auteur!D143</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="128" t="n">
+      <c r="A79" s="124" t="n">
         <v>13</v>
       </c>
-      <c r="B79" s="129"/>
-      <c r="C79" s="129"/>
-      <c r="D79" s="129"/>
-      <c r="E79" s="129"/>
-      <c r="F79" s="130" t="n">
+      <c r="B79" s="125"/>
+      <c r="C79" s="125"/>
+      <c r="D79" s="125"/>
+      <c r="E79" s="125"/>
+      <c r="F79" s="126" t="n">
         <v>144</v>
       </c>
-      <c r="G79" s="129" t="str">
+      <c r="G79" s="125" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F79</f>
         <v>Auteur!C144</v>
       </c>
-      <c r="H79" s="131" t="str">
+      <c r="H79" s="127" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F79</f>
         <v>Auteur!D144</v>
       </c>
@@ -8368,7 +8409,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D80</f>
         <v>Auteur!D151</v>
       </c>
-      <c r="F80" s="118" t="n">
+      <c r="F80" s="114" t="n">
         <v>153</v>
       </c>
       <c r="G80" s="2" t="str">
@@ -8552,7 +8593,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D90</f>
         <v>Auteur!D165</v>
       </c>
-      <c r="F90" s="118" t="n">
+      <c r="F90" s="114" t="n">
         <v>167</v>
       </c>
       <c r="G90" s="2" t="str">

</xml_diff>

<commit_message>
Export ZIP, accès public marqueur, refonte fichiers Volume et docs
- Marqueur, guide et test-sons accessibles sans mot de passe (admin seul protégé)
- Export sauvegarde ZIP : endpoint public /api/sauvegarde-zip (marqueur) + admin /api/admin/export-zip
- Bannière de sauvegarde après fin de partie dans le marqueur
- Correction affichage post-partie : bouton centré, joueurs masqués après terminer
- index.js : tous les fichiers admin dans fichiersAdmin (copier si absent), suppression fichiersGit
- questions.json et thèmes.json retirés du suivi git (re-ajoutés au .gitignore)
- Éliminatoires : affichage équipe questionnaire et animateur sur chaque carte
- guide-animateur.html : table fichiers à jour, section sauvegarde ZIP, import historique corrigé
- docs.html : gabarit questionnaire 3 mis à jour (nom de fichier fixe)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/ressources/2025-2026/gabarit-q3.xlsx
+++ b/public/ressources/2025-2026/gabarit-q3.xlsx
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="149">
   <si>
     <r>
       <rPr>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t xml:space="preserve">Série 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Libre</t>
   </si>
   <si>
     <t xml:space="preserve">Choix d'associations</t>
@@ -1849,9 +1852,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2521080</xdr:colOff>
+      <xdr:colOff>2520360</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>120960</xdr:rowOff>
+      <xdr:rowOff>120240</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1861,7 +1864,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="681840" y="325800"/>
-          <a:ext cx="2714760" cy="1442880"/>
+          <a:ext cx="2714040" cy="1442160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2001,9 +2004,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>467640</xdr:colOff>
+      <xdr:colOff>466920</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>178200</xdr:rowOff>
+      <xdr:rowOff>177480</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2013,7 +2016,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9114120" y="314280"/>
-          <a:ext cx="1580040" cy="368640"/>
+          <a:ext cx="1579320" cy="367920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2073,7 +2076,7 @@
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>Version 2.1</a:t>
+            <a:t>Version 2.2</a:t>
           </a:r>
           <a:endParaRPr lang="fr-CA" sz="1000" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -2093,10 +2096,10 @@
       <xdr:rowOff>163800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1080</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>634680</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>180000</xdr:rowOff>
+      <xdr:rowOff>179280</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2106,7 +2109,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="478080"/>
-          <a:ext cx="635400" cy="1349640"/>
+          <a:ext cx="634680" cy="1348920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3644,14 +3647,14 @@
         <v>49</v>
       </c>
       <c r="D124" s="13" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="E124" s="23"/>
     </row>
     <row r="125" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B125" s="14"/>
       <c r="C125" s="15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D125" s="16" t="str">
         <f aca="false">C128 &amp; " / " &amp;C139</f>
@@ -3662,7 +3665,7 @@
     <row r="126" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="29"/>
       <c r="C126" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D126" s="18"/>
       <c r="E126" s="23"/>
@@ -3670,7 +3673,7 @@
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="75"/>
       <c r="C127" s="45" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D127" s="76"/>
       <c r="E127" s="23"/>
@@ -3678,7 +3681,7 @@
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="77"/>
       <c r="C128" s="78" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D128" s="79"/>
       <c r="E128" s="23"/>
@@ -3686,7 +3689,7 @@
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B129" s="77"/>
       <c r="C129" s="78" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D129" s="79"/>
       <c r="E129" s="23"/>
@@ -3737,7 +3740,7 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="81" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C134" s="71"/>
       <c r="D134" s="72"/>
@@ -3745,7 +3748,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B135" s="82" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C135" s="32"/>
       <c r="D135" s="22"/>
@@ -3753,7 +3756,7 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B136" s="82" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C136" s="32"/>
       <c r="D136" s="22"/>
@@ -3761,7 +3764,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="83" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C137" s="26"/>
       <c r="D137" s="27"/>
@@ -3770,7 +3773,7 @@
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B138" s="77"/>
       <c r="C138" s="45" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D138" s="79"/>
       <c r="E138" s="23"/>
@@ -3778,7 +3781,7 @@
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B139" s="77"/>
       <c r="C139" s="78" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D139" s="79"/>
       <c r="E139" s="23"/>
@@ -3786,7 +3789,7 @@
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="77"/>
       <c r="C140" s="78" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D140" s="84"/>
       <c r="E140" s="23"/>
@@ -3837,7 +3840,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B145" s="81" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C145" s="71"/>
       <c r="D145" s="72"/>
@@ -3845,7 +3848,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B146" s="82" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C146" s="32"/>
       <c r="D146" s="22"/>
@@ -3853,7 +3856,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B147" s="82" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C147" s="32"/>
       <c r="D147" s="22"/>
@@ -3861,7 +3864,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="83" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C148" s="26"/>
       <c r="D148" s="27"/>
@@ -3876,17 +3879,17 @@
     <row r="150" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B150" s="11"/>
       <c r="C150" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D150" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E150" s="23"/>
     </row>
     <row r="151" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B151" s="14"/>
       <c r="C151" s="15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D151" s="16"/>
       <c r="E151" s="23"/>
@@ -3894,7 +3897,7 @@
     <row r="152" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B152" s="29"/>
       <c r="C152" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D152" s="18"/>
       <c r="E152" s="23"/>
@@ -4018,17 +4021,17 @@
     <row r="164" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B164" s="11"/>
       <c r="C164" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D164" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E164" s="23"/>
     </row>
     <row r="165" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B165" s="14"/>
       <c r="C165" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D165" s="16"/>
       <c r="E165" s="23"/>
@@ -4036,7 +4039,7 @@
     <row r="166" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B166" s="29"/>
       <c r="C166" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D166" s="18"/>
       <c r="E166" s="23"/>
@@ -4081,7 +4084,7 @@
     <mergeCell ref="B123:D123"/>
     <mergeCell ref="B163:D163"/>
   </mergeCells>
-  <conditionalFormatting sqref="D60 D91 D98 D124">
+  <conditionalFormatting sqref="D60 D91 D98">
     <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="-- Choisir un thème --" dxfId="0">
       <formula>NOT(ISERROR(SEARCH("-- Choisir un thème --",D60)))</formula>
     </cfRule>
@@ -4091,21 +4094,17 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D60" type="list">
-      <formula1>"-- Choisir un thème --,Arts et littérature,Cinéma et télévision,Musique"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D98" type="list">
-      <formula1>"-- Choisir un thème --,Actualité,Histoire et société,Langue"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
+  <dataValidations count="3">
     <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D91" type="list">
       <formula1>"-- Choisir un thème --,Actualité,Arts et littérature,Cinéma et télévision,Géographie,Histoire et société,Langue,Musique,Sciences,Sports et loisirs"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D124" type="list">
-      <formula1>"-- Choisir un thème --,Divers,Actualité,Arts et littérature,Cinéma et télévision,Géographie,Histoire et société,Langue,Musique,Sciences,Sports et loisirs"</formula1>
+    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D60" type="list">
+      <formula1>"-- Choisir un thème --,Actualité,Histoire et société,Langue,"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Vous devez choisir l'un des thèmes prescrits." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D98" type="list">
+      <formula1>"-- Choisir un thème --,Géographie,Sciences,Sports et loisirs"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4148,21 +4147,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="88" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="89" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B2" s="89" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C2" s="89" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D2" s="89" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4395,7 +4394,7 @@
       </c>
       <c r="C15" s="2" t="str">
         <f aca="true">INDIRECT(Adresses!C72)</f>
-        <v>-- Choisir un thème --</v>
+        <v>Libre</v>
       </c>
       <c r="D15" s="2" t="str">
         <f aca="true">IF(INDIRECT(Adresses!E72)&lt;&gt;0,INDIRECT(Adresses!E72),"")</f>
@@ -4440,24 +4439,24 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="88" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="89" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B20" s="89" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C20" s="89" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D20" s="89" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E20" s="89" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5797,7 +5796,7 @@
         <v>13</v>
       </c>
       <c r="C84" s="90" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D84" s="90" t="str">
         <f aca="false">Auteur!C129</f>
@@ -5898,7 +5897,7 @@
         <v>13</v>
       </c>
       <c r="C89" s="90" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D89" s="90" t="str">
         <f aca="false">Auteur!C140</f>
@@ -6416,11 +6415,11 @@
       </c>
       <c r="B3" s="94"/>
       <c r="C3" s="95" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D3" s="95"/>
       <c r="G3" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6429,11 +6428,11 @@
       </c>
       <c r="B4" s="94"/>
       <c r="C4" s="95" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D4" s="95"/>
       <c r="G4" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6442,13 +6441,13 @@
       </c>
       <c r="B5" s="94"/>
       <c r="C5" s="95" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D5" s="95"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="94" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B6" s="94"/>
       <c r="C6" s="95"/>
@@ -6456,7 +6455,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="94" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B7" s="94"/>
       <c r="C7" s="95"/>
@@ -6464,7 +6463,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="96" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B8" s="96"/>
       <c r="C8" s="97"/>
@@ -6478,7 +6477,7 @@
     </row>
     <row r="10" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="98" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B10" s="98"/>
       <c r="C10" s="98"/>
@@ -6492,11 +6491,11 @@
     </row>
     <row r="12" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="100" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B12" s="100"/>
       <c r="C12" s="100" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D12" s="101"/>
     </row>
@@ -6506,10 +6505,10 @@
       </c>
       <c r="B13" s="102"/>
       <c r="C13" s="103" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D13" s="104" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6551,11 +6550,11 @@
         <v>2</v>
       </c>
       <c r="B18" s="107" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C18" s="107"/>
       <c r="D18" s="108" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6563,11 +6562,11 @@
         <v>3</v>
       </c>
       <c r="B19" s="107" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C19" s="107"/>
       <c r="D19" s="108" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6575,11 +6574,11 @@
         <v>4</v>
       </c>
       <c r="B20" s="107" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C20" s="107"/>
       <c r="D20" s="108" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6595,11 +6594,11 @@
         <v>1</v>
       </c>
       <c r="B22" s="107" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C22" s="107"/>
       <c r="D22" s="108" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6607,11 +6606,11 @@
         <v>2</v>
       </c>
       <c r="B23" s="107" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C23" s="107"/>
       <c r="D23" s="108" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6619,11 +6618,11 @@
         <v>3</v>
       </c>
       <c r="B24" s="107" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C24" s="107"/>
       <c r="D24" s="108" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6631,11 +6630,11 @@
         <v>4</v>
       </c>
       <c r="B25" s="107" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C25" s="107"/>
       <c r="D25" s="108" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6646,7 +6645,7 @@
     </row>
     <row r="27" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="98" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B27" s="98"/>
       <c r="C27" s="98"/>
@@ -6660,19 +6659,19 @@
     </row>
     <row r="29" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="100" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B29" s="100"/>
       <c r="C29" s="109" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D29" s="110" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="111" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B30" s="111"/>
       <c r="C30" s="109"/>
@@ -6683,11 +6682,11 @@
         <v>1</v>
       </c>
       <c r="B31" s="107" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C31" s="107"/>
       <c r="D31" s="108" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6695,11 +6694,11 @@
         <v>2</v>
       </c>
       <c r="B32" s="107" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C32" s="107"/>
       <c r="D32" s="108" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6707,11 +6706,11 @@
         <v>3</v>
       </c>
       <c r="B33" s="107" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C33" s="107"/>
       <c r="D33" s="108" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6719,11 +6718,11 @@
         <v>4</v>
       </c>
       <c r="B34" s="107" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C34" s="107"/>
       <c r="D34" s="108" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6731,11 +6730,11 @@
         <v>5</v>
       </c>
       <c r="B35" s="107" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C35" s="107"/>
       <c r="D35" s="108" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6746,19 +6745,19 @@
     </row>
     <row r="37" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="100" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B37" s="100"/>
       <c r="C37" s="109" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D37" s="110" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="111" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B38" s="111"/>
       <c r="C38" s="109"/>
@@ -6769,11 +6768,11 @@
         <v>1</v>
       </c>
       <c r="B39" s="107" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C39" s="107"/>
       <c r="D39" s="108" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6781,11 +6780,11 @@
         <v>2</v>
       </c>
       <c r="B40" s="107" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C40" s="107"/>
       <c r="D40" s="108" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6793,11 +6792,11 @@
         <v>3</v>
       </c>
       <c r="B41" s="107" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C41" s="107"/>
       <c r="D41" s="108" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6805,11 +6804,11 @@
         <v>4</v>
       </c>
       <c r="B42" s="107" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C42" s="107"/>
       <c r="D42" s="108" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6817,17 +6816,17 @@
         <v>5</v>
       </c>
       <c r="B43" s="112" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C43" s="112"/>
       <c r="D43" s="113" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="77.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="107"/>
       <c r="B44" s="106" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C44" s="106"/>
       <c r="D44" s="113"/>
@@ -6919,73 +6918,73 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="114" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="115" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B8" s="116" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C8" s="116" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D8" s="116" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E8" s="116" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F8" s="116" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G8" s="116" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H8" s="116" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Mise a jour du gabarit pour avoir les questions sup.
</commit_message>
<xml_diff>
--- a/public/ressources/2025-2026/gabarit-q3.xlsx
+++ b/public/ressources/2025-2026/gabarit-q3.xlsx
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="152">
   <si>
     <r>
       <rPr>
@@ -334,6 +334,33 @@
     <t xml:space="preserve">Poser une question demandant une réponse simple, pour éviter les ambiguïtés.</t>
   </si>
   <si>
+    <t xml:space="preserve">Série 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Questions supplémentaires</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Séries seulement : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Viser des questions courtes couvrant un maximum de thèmes différents.</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">tblThèmes</t>
   </si>
   <si>
@@ -633,7 +660,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy/mm/dd"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -767,6 +794,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color rgb="FF339966"/>
       <name val="Arial"/>
@@ -834,7 +868,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -845,6 +879,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor rgb="FF993300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7B59"/>
+        <bgColor rgb="FFFF6600"/>
       </patternFill>
     </fill>
     <fill>
@@ -1278,7 +1318,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="129">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1631,11 +1671,15 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="20" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="13" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="13" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1671,7 +1715,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1739,11 +1783,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="46" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="46" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="47" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="47" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1767,7 +1811,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1783,7 +1827,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="52" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="52" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1838,6 +1882,66 @@
       </fill>
     </dxf>
   </dxfs>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF7B59"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1852,9 +1956,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2520360</xdr:colOff>
+      <xdr:colOff>2519640</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>120240</xdr:rowOff>
+      <xdr:rowOff>119520</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1864,7 +1968,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="681840" y="325800"/>
-          <a:ext cx="2714040" cy="1442160"/>
+          <a:ext cx="2713320" cy="1441440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2004,9 +2108,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>466920</xdr:colOff>
+      <xdr:colOff>466200</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>177480</xdr:rowOff>
+      <xdr:rowOff>176760</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2016,7 +2120,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9114120" y="314280"/>
-          <a:ext cx="1579320" cy="367920"/>
+          <a:ext cx="1578600" cy="367200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2076,7 +2180,7 @@
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>Version 2.2</a:t>
+            <a:t>Version 3.0</a:t>
           </a:r>
           <a:endParaRPr lang="fr-CA" sz="1000" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -2097,9 +2201,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>634680</xdr:colOff>
+      <xdr:colOff>633960</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>179280</xdr:rowOff>
+      <xdr:rowOff>178560</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2109,7 +2213,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="478080"/>
-          <a:ext cx="634680" cy="1348920"/>
+          <a:ext cx="633960" cy="1348200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2457,7 +2561,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I167"/>
+  <dimension ref="A1:I178"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -2679,7 +2783,7 @@
       <c r="D25" s="16"/>
       <c r="E25" s="23"/>
     </row>
-    <row r="26" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="29"/>
       <c r="C26" s="17" t="s">
         <v>17</v>
@@ -2766,7 +2870,7 @@
       <c r="D34" s="16"/>
       <c r="E34" s="23"/>
     </row>
-    <row r="35" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="29"/>
       <c r="C35" s="17" t="s">
         <v>21</v>
@@ -2919,7 +3023,7 @@
       <c r="D50" s="47"/>
       <c r="E50" s="23"/>
     </row>
-    <row r="51" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="11"/>
       <c r="C51" s="12" t="s">
         <v>25</v>
@@ -2937,7 +3041,7 @@
       <c r="D52" s="16"/>
       <c r="E52" s="23"/>
     </row>
-    <row r="53" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="28.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="29"/>
       <c r="C53" s="17" t="s">
         <v>28</v>
@@ -3032,7 +3136,7 @@
       <c r="H61" s="51"/>
       <c r="I61" s="52"/>
     </row>
-    <row r="62" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="29"/>
       <c r="C62" s="17" t="s">
         <v>34</v>
@@ -3342,7 +3446,7 @@
       <c r="D92" s="16"/>
       <c r="E92" s="23"/>
     </row>
-    <row r="93" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="29"/>
       <c r="C93" s="17" t="s">
         <v>41</v>
@@ -3483,7 +3587,7 @@
       <c r="D107" s="63"/>
       <c r="E107" s="23"/>
     </row>
-    <row r="108" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="29"/>
       <c r="C108" s="17" t="s">
         <v>17</v>
@@ -3572,7 +3676,7 @@
       <c r="D116" s="63"/>
       <c r="E116" s="23"/>
     </row>
-    <row r="117" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="29"/>
       <c r="C117" s="17" t="s">
         <v>17</v>
@@ -3662,7 +3766,7 @@
       </c>
       <c r="E125" s="23"/>
     </row>
-    <row r="126" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="29"/>
       <c r="C126" s="17" t="s">
         <v>52</v>
@@ -4054,6 +4158,78 @@
       <c r="C167" s="71"/>
       <c r="D167" s="72"/>
       <c r="E167" s="23"/>
+    </row>
+    <row r="169" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B169" s="11"/>
+      <c r="C169" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D169" s="13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B170" s="14"/>
+      <c r="C170" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D170" s="16"/>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B171" s="29"/>
+      <c r="C171" s="88" t="s">
+        <v>73</v>
+      </c>
+      <c r="D171" s="18"/>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B172" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C172" s="71"/>
+      <c r="D172" s="72"/>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B173" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C173" s="32"/>
+      <c r="D173" s="33"/>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B174" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C174" s="32"/>
+      <c r="D174" s="33"/>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B175" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C175" s="32"/>
+      <c r="D175" s="33"/>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B176" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C176" s="32"/>
+      <c r="D176" s="33"/>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B177" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C177" s="32"/>
+      <c r="D177" s="33"/>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B178" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="C178" s="80"/>
+      <c r="D178" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -4130,7 +4306,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:IT111"/>
+  <dimension ref="A1:IT119"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="14.86"/>
@@ -4146,22 +4322,22 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="88" t="s">
-        <v>71</v>
+      <c r="A1" s="89" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="89" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="89" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="89" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="89" t="s">
+      <c r="A2" s="90" t="s">
         <v>75</v>
+      </c>
+      <c r="B2" s="90" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="90" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="90" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4198,10 +4374,10 @@
         <f aca="true">IF(INDIRECT(Adresses!E17)&lt;&gt;0,INDIRECT(Adresses!E17),"")</f>
         <v/>
       </c>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90"/>
+      <c r="F4" s="91"/>
+      <c r="G4" s="91"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="91"/>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
@@ -4437,1493 +4613,1491 @@
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="88" t="s">
+    <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <f aca="false">B17+1</f>
+        <v>16</v>
+      </c>
+      <c r="C18" s="2" t="str">
+        <f aca="true">INDIRECT(Adresses!C91)</f>
+        <v>Divers</v>
+      </c>
+      <c r="D18" s="2" t="str">
+        <f aca="true">IF(INDIRECT(Adresses!E91)&lt;&gt;0,INDIRECT(Adresses!E91),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="89" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="90" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" s="90" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="89" t="s">
-        <v>72</v>
-      </c>
-      <c r="B20" s="89" t="s">
-        <v>73</v>
-      </c>
-      <c r="C20" s="89" t="s">
-        <v>77</v>
-      </c>
-      <c r="D20" s="89" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="89" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B21" s="90" t="n">
+      <c r="C21" s="90" t="s">
+        <v>80</v>
+      </c>
+      <c r="D21" s="90" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" s="90" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B22" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="90" t="n">
+      <c r="C22" s="91" t="n">
         <f aca="false">Auteur!B14</f>
         <v>1</v>
       </c>
-      <c r="D21" s="90" t="n">
+      <c r="D22" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G9)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="90" t="n">
+      <c r="E22" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H9)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B22" s="2" t="n">
+    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="90" t="n">
+      <c r="C23" s="91" t="n">
         <f aca="false">Auteur!B15</f>
         <v>2</v>
       </c>
-      <c r="D22" s="90" t="n">
+      <c r="D23" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G10)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="90" t="n">
+      <c r="E23" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H10)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B23" s="2" t="n">
+    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="90" t="n">
+      <c r="C24" s="91" t="n">
         <f aca="false">Auteur!B16</f>
         <v>3</v>
       </c>
-      <c r="D23" s="90" t="n">
+      <c r="D24" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G11)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="90" t="n">
+      <c r="E24" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H11)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B24" s="2" t="n">
+    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="90" t="n">
+      <c r="C25" s="91" t="n">
         <f aca="false">Auteur!B17</f>
         <v>4</v>
       </c>
-      <c r="D24" s="90" t="n">
+      <c r="D25" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G12)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="90" t="n">
+      <c r="E25" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H12)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B25" s="2" t="n">
+    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C25" s="90" t="n">
+      <c r="C26" s="91" t="n">
         <f aca="false">Auteur!B19</f>
         <v>5</v>
       </c>
-      <c r="D25" s="90" t="n">
+      <c r="D26" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G13)</f>
         <v>0</v>
       </c>
-      <c r="E25" s="90" t="n">
+      <c r="E26" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H13)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B26" s="2" t="n">
+    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C26" s="90" t="n">
+      <c r="C27" s="91" t="n">
         <f aca="false">Auteur!B20</f>
         <v>6</v>
       </c>
-      <c r="D26" s="90" t="n">
+      <c r="D27" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G14)</f>
         <v>0</v>
       </c>
-      <c r="E26" s="90" t="n">
+      <c r="E27" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H14)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B27" s="2" t="n">
+    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C27" s="90" t="n">
+      <c r="C28" s="91" t="n">
         <f aca="false">Auteur!B21</f>
         <v>7</v>
       </c>
-      <c r="D27" s="90" t="n">
+      <c r="D28" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G15)</f>
         <v>0</v>
       </c>
-      <c r="E27" s="90" t="n">
+      <c r="E28" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H15)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B28" s="2" t="n">
+    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C28" s="90" t="n">
+      <c r="C29" s="91" t="n">
         <f aca="false">Auteur!B22</f>
         <v>8</v>
       </c>
-      <c r="D28" s="90" t="n">
+      <c r="D29" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G16)</f>
         <v>0</v>
       </c>
-      <c r="E28" s="90" t="n">
+      <c r="E29" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H16)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B29" s="2" t="n">
+    <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C29" s="90" t="n">
+      <c r="C30" s="91" t="n">
         <f aca="false">Auteur!B27</f>
         <v>1</v>
       </c>
-      <c r="D29" s="90" t="n">
+      <c r="D30" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G17)</f>
         <v>0</v>
       </c>
-      <c r="E29" s="90" t="n">
+      <c r="E30" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H17)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B30" s="2" t="n">
+    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B31" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C30" s="90" t="n">
+      <c r="C31" s="91" t="n">
         <f aca="false">Auteur!B28</f>
         <v>2</v>
       </c>
-      <c r="D30" s="90" t="n">
+      <c r="D31" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G18)</f>
         <v>0</v>
       </c>
-      <c r="E30" s="90" t="n">
+      <c r="E31" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H18)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B31" s="2" t="n">
+    <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B32" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C31" s="90" t="n">
+      <c r="C32" s="91" t="n">
         <f aca="false">Auteur!B29</f>
         <v>3</v>
       </c>
-      <c r="D31" s="90" t="n">
+      <c r="D32" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G19)</f>
         <v>0</v>
       </c>
-      <c r="E31" s="90" t="n">
+      <c r="E32" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H19)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B32" s="2" t="n">
+    <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="90" t="n">
+      <c r="C33" s="91" t="n">
         <f aca="false">Auteur!B30</f>
         <v>4</v>
       </c>
-      <c r="D32" s="90" t="n">
+      <c r="D33" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G20)</f>
         <v>0</v>
       </c>
-      <c r="E32" s="90" t="n">
+      <c r="E33" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H20)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B33" s="2" t="n">
+    <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B34" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C33" s="90" t="n">
+      <c r="C34" s="91" t="n">
         <f aca="false">Auteur!B31</f>
         <v>5</v>
       </c>
-      <c r="D33" s="90" t="n">
+      <c r="D34" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G21)</f>
         <v>0</v>
       </c>
-      <c r="E33" s="90" t="n">
+      <c r="E34" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H21)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B34" s="2" t="n">
+    <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B35" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C34" s="90" t="n">
+      <c r="C35" s="91" t="n">
         <f aca="false">Auteur!B36</f>
         <v>1</v>
       </c>
-      <c r="D34" s="90" t="n">
+      <c r="D35" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G22)</f>
         <v>0</v>
       </c>
-      <c r="E34" s="90" t="n">
+      <c r="E35" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H22)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B35" s="2" t="n">
+    <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B36" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C35" s="90" t="n">
+      <c r="C36" s="91" t="n">
         <f aca="false">Auteur!B37</f>
         <v>2</v>
       </c>
-      <c r="D35" s="90" t="n">
+      <c r="D36" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G23)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="90" t="n">
+      <c r="E36" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H23)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B36" s="2" t="n">
+    <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B37" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C36" s="90" t="n">
+      <c r="C37" s="91" t="n">
         <f aca="false">Auteur!B38</f>
         <v>3</v>
       </c>
-      <c r="D36" s="90" t="n">
+      <c r="D37" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G24)</f>
         <v>0</v>
       </c>
-      <c r="E36" s="90" t="n">
+      <c r="E37" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H24)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B37" s="2" t="n">
+    <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B38" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C37" s="90" t="n">
+      <c r="C38" s="91" t="n">
         <f aca="false">Auteur!B39</f>
         <v>4</v>
       </c>
-      <c r="D37" s="90" t="n">
+      <c r="D38" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G25)</f>
         <v>0</v>
       </c>
-      <c r="E37" s="90" t="n">
+      <c r="E38" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H25)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B38" s="2" t="n">
+    <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C38" s="90" t="n">
+      <c r="C39" s="91" t="n">
         <f aca="false">Auteur!B40</f>
         <v>5</v>
       </c>
-      <c r="D38" s="90" t="n">
+      <c r="D39" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G26)</f>
         <v>0</v>
       </c>
-      <c r="E38" s="90" t="n">
+      <c r="E39" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H26)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B39" s="2" t="n">
+    <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B40" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C39" s="90" t="n">
+      <c r="C40" s="91" t="n">
         <f aca="false">Auteur!B45</f>
         <v>1</v>
       </c>
-      <c r="D39" s="90" t="n">
+      <c r="D40" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G27)</f>
         <v>0</v>
       </c>
-      <c r="E39" s="90" t="n">
+      <c r="E40" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H27)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B40" s="2" t="n">
+    <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B41" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C40" s="90" t="n">
+      <c r="C41" s="91" t="n">
         <f aca="false">Auteur!B46</f>
         <v>2</v>
       </c>
-      <c r="D40" s="90" t="n">
+      <c r="D41" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G28)</f>
         <v>0</v>
       </c>
-      <c r="E40" s="90" t="n">
+      <c r="E41" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H28)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B41" s="2" t="n">
+    <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B42" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C41" s="90" t="n">
+      <c r="C42" s="91" t="n">
         <f aca="false">Auteur!B47</f>
         <v>3</v>
       </c>
-      <c r="D41" s="90" t="n">
+      <c r="D42" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G29)</f>
         <v>0</v>
       </c>
-      <c r="E41" s="90" t="n">
+      <c r="E42" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H29)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B42" s="2" t="n">
+    <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B43" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C42" s="90" t="n">
+      <c r="C43" s="91" t="n">
         <f aca="false">Auteur!B48</f>
         <v>4</v>
       </c>
-      <c r="D42" s="90" t="n">
+      <c r="D43" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G30)</f>
         <v>0</v>
       </c>
-      <c r="E42" s="90" t="n">
+      <c r="E43" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H30)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B43" s="2" t="n">
+    <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B44" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C43" s="90" t="n">
+      <c r="C44" s="91" t="n">
         <f aca="false">Auteur!B49</f>
         <v>5</v>
       </c>
-      <c r="D43" s="90" t="n">
+      <c r="D44" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G31)</f>
         <v>0</v>
       </c>
-      <c r="E43" s="90" t="n">
+      <c r="E44" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H31)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B44" s="2" t="n">
+    <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B45" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C44" s="90" t="n">
+      <c r="C45" s="91" t="n">
         <f aca="false">Auteur!B54</f>
         <v>1</v>
       </c>
-      <c r="D44" s="90" t="n">
+      <c r="D45" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G32)</f>
         <v>0</v>
       </c>
-      <c r="E44" s="90" t="n">
+      <c r="E45" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H32)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B45" s="2" t="n">
+    <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B46" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C45" s="90" t="n">
+      <c r="C46" s="91" t="n">
         <f aca="false">Auteur!B55</f>
         <v>2</v>
       </c>
-      <c r="D45" s="90" t="n">
+      <c r="D46" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G33)</f>
         <v>0</v>
       </c>
-      <c r="E45" s="90" t="n">
+      <c r="E46" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H33)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B46" s="2" t="n">
+    <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B47" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C46" s="90" t="n">
+      <c r="C47" s="91" t="n">
         <f aca="false">Auteur!B56</f>
         <v>3</v>
       </c>
-      <c r="D46" s="90" t="n">
+      <c r="D47" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G34)</f>
         <v>0</v>
       </c>
-      <c r="E46" s="90" t="n">
+      <c r="E47" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H34)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B47" s="2" t="n">
+    <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B48" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C47" s="90" t="n">
+      <c r="C48" s="91" t="n">
         <f aca="false">Auteur!B57</f>
         <v>4</v>
       </c>
-      <c r="D47" s="90" t="n">
+      <c r="D48" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G35)</f>
         <v>0</v>
       </c>
-      <c r="E47" s="90" t="n">
+      <c r="E48" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H35)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B48" s="2" t="n">
+    <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B49" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C48" s="90" t="n">
+      <c r="C49" s="91" t="n">
         <f aca="false">Auteur!B58</f>
         <v>5</v>
       </c>
-      <c r="D48" s="90" t="n">
+      <c r="D49" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G36)</f>
         <v>0</v>
       </c>
-      <c r="E48" s="90" t="n">
+      <c r="E49" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H36)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B49" s="2" t="n">
+    <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B50" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C49" s="90" t="n">
+      <c r="C50" s="91" t="n">
         <f aca="false">Auteur!B64</f>
         <v>1</v>
       </c>
-      <c r="D49" s="90" t="n">
+      <c r="D50" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G37)</f>
         <v>0</v>
       </c>
-      <c r="E49" s="90" t="n">
+      <c r="E50" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H37)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B50" s="2" t="n">
+    <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B51" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C50" s="90" t="n">
+      <c r="C51" s="91" t="n">
         <f aca="false">Auteur!B65</f>
         <v>2</v>
       </c>
-      <c r="D50" s="90" t="n">
+      <c r="D51" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G38)</f>
         <v>0</v>
       </c>
-      <c r="E50" s="90" t="n">
+      <c r="E51" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H38)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B51" s="2" t="n">
+    <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B52" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C51" s="90" t="n">
+      <c r="C52" s="91" t="n">
         <f aca="false">Auteur!B66</f>
         <v>3</v>
       </c>
-      <c r="D51" s="90" t="n">
+      <c r="D52" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G39)</f>
         <v>0</v>
       </c>
-      <c r="E51" s="90" t="n">
+      <c r="E52" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H39)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B52" s="2" t="n">
+    <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B53" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C52" s="90" t="n">
+      <c r="C53" s="91" t="n">
         <f aca="false">Auteur!B67</f>
         <v>4</v>
       </c>
-      <c r="D52" s="90" t="n">
+      <c r="D53" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G40)</f>
         <v>0</v>
       </c>
-      <c r="E52" s="90" t="n">
+      <c r="E53" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H40)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B53" s="2" t="n">
+    <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B54" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C53" s="90" t="n">
+      <c r="C54" s="91" t="n">
         <f aca="false">Auteur!B68</f>
         <v>5</v>
       </c>
-      <c r="D53" s="90" t="n">
+      <c r="D54" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G41)</f>
         <v>0</v>
       </c>
-      <c r="E53" s="90" t="n">
+      <c r="E54" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H41)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B54" s="2" t="n">
+    <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B55" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C54" s="90" t="n">
+      <c r="C55" s="91" t="n">
         <f aca="false">Auteur!B69</f>
         <v>6</v>
       </c>
-      <c r="D54" s="90" t="n">
+      <c r="D55" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G42)</f>
         <v>0</v>
       </c>
-      <c r="E54" s="90" t="n">
+      <c r="E55" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H42)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B55" s="2" t="n">
+    <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B56" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C55" s="90" t="n">
+      <c r="C56" s="91" t="n">
         <f aca="false">Auteur!B70</f>
         <v>7</v>
       </c>
-      <c r="D55" s="90" t="n">
+      <c r="D56" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G43)</f>
         <v>0</v>
       </c>
-      <c r="E55" s="90" t="n">
+      <c r="E56" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H43)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B56" s="2" t="n">
+    <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B57" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C56" s="90" t="n">
+      <c r="C57" s="91" t="n">
         <f aca="false">Auteur!B71</f>
         <v>8</v>
       </c>
-      <c r="D56" s="90" t="n">
+      <c r="D57" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G44)</f>
         <v>0</v>
       </c>
-      <c r="E56" s="90" t="n">
+      <c r="E57" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H44)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B57" s="2" t="n">
+    <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B58" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C57" s="90" t="n">
+      <c r="C58" s="91" t="n">
         <f aca="false">Auteur!B76</f>
         <v>1</v>
       </c>
-      <c r="D57" s="90" t="n">
+      <c r="D58" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G45)</f>
         <v>0</v>
       </c>
-      <c r="E57" s="90" t="n">
+      <c r="E58" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H45)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B58" s="2" t="n">
+    <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B59" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C58" s="90" t="n">
+      <c r="C59" s="91" t="n">
         <f aca="false">Auteur!B77</f>
         <v>2</v>
       </c>
-      <c r="D58" s="90" t="n">
+      <c r="D59" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G46)</f>
         <v>0</v>
       </c>
-      <c r="E58" s="90" t="n">
+      <c r="E59" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H46)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B59" s="2" t="n">
+    <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B60" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C59" s="90" t="n">
+      <c r="C60" s="91" t="n">
         <f aca="false">Auteur!B78</f>
         <v>3</v>
       </c>
-      <c r="D59" s="90" t="n">
+      <c r="D60" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G47)</f>
         <v>0</v>
       </c>
-      <c r="E59" s="90" t="n">
+      <c r="E60" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H47)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B60" s="2" t="n">
+    <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B61" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C60" s="90" t="n">
+      <c r="C61" s="91" t="n">
         <f aca="false">Auteur!B79</f>
         <v>4</v>
       </c>
-      <c r="D60" s="90" t="n">
+      <c r="D61" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G48)</f>
         <v>0</v>
       </c>
-      <c r="E60" s="90" t="n">
+      <c r="E61" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H48)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B61" s="2" t="n">
+    <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B62" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C61" s="90" t="n">
+      <c r="C62" s="91" t="n">
         <f aca="false">Auteur!B80</f>
         <v>5</v>
       </c>
-      <c r="D61" s="90" t="n">
+      <c r="D62" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G49)</f>
         <v>0</v>
       </c>
-      <c r="E61" s="90" t="n">
+      <c r="E62" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H49)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B62" s="2" t="n">
+    <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B63" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C62" s="90" t="n">
+      <c r="C63" s="91" t="n">
         <f aca="false">Auteur!B85</f>
         <v>1</v>
       </c>
-      <c r="D62" s="90" t="n">
+      <c r="D63" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G50)</f>
         <v>0</v>
       </c>
-      <c r="E62" s="90" t="n">
+      <c r="E63" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H50)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B63" s="2" t="n">
+    <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B64" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C63" s="90" t="n">
+      <c r="C64" s="91" t="n">
         <f aca="false">Auteur!B86</f>
         <v>2</v>
       </c>
-      <c r="D63" s="90" t="n">
+      <c r="D64" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G51)</f>
         <v>0</v>
       </c>
-      <c r="E63" s="90" t="n">
+      <c r="E64" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H51)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B64" s="2" t="n">
+    <row r="65" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B65" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C64" s="90" t="n">
+      <c r="C65" s="91" t="n">
         <f aca="false">Auteur!B87</f>
         <v>3</v>
       </c>
-      <c r="D64" s="90" t="n">
+      <c r="D65" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G52)</f>
         <v>0</v>
       </c>
-      <c r="E64" s="90" t="n">
+      <c r="E65" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H52)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B65" s="2" t="n">
+    <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B66" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C65" s="90" t="n">
+      <c r="C66" s="91" t="n">
         <f aca="false">Auteur!B88</f>
         <v>4</v>
       </c>
-      <c r="D65" s="90" t="n">
+      <c r="D66" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G53)</f>
         <v>0</v>
       </c>
-      <c r="E65" s="90" t="n">
+      <c r="E66" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H53)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B66" s="2" t="n">
+    <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B67" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C66" s="90" t="n">
+      <c r="C67" s="91" t="n">
         <f aca="false">Auteur!B89</f>
         <v>5</v>
       </c>
-      <c r="D66" s="90" t="n">
+      <c r="D67" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G54)</f>
         <v>0</v>
       </c>
-      <c r="E66" s="90" t="n">
+      <c r="E67" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H54)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B67" s="2" t="n">
+    <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B68" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C67" s="90" t="n">
+      <c r="C68" s="91" t="n">
         <f aca="false">Auteur!B94</f>
         <v>1</v>
       </c>
-      <c r="D67" s="90" t="n">
+      <c r="D68" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G55)</f>
         <v>0</v>
       </c>
-      <c r="E67" s="90" t="n">
+      <c r="E68" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H55)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B68" s="2" t="n">
+    <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B69" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C68" s="90" t="n">
+      <c r="C69" s="91" t="n">
         <f aca="false">Auteur!B95</f>
         <v>2</v>
       </c>
-      <c r="D68" s="90" t="n">
+      <c r="D69" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G56)</f>
         <v>0</v>
       </c>
-      <c r="E68" s="90" t="n">
+      <c r="E69" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H56)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B69" s="2" t="n">
+    <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B70" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C69" s="90" t="n">
+      <c r="C70" s="91" t="n">
         <f aca="false">Auteur!B96</f>
         <v>3</v>
       </c>
-      <c r="D69" s="90" t="n">
+      <c r="D70" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G57)</f>
         <v>0</v>
       </c>
-      <c r="E69" s="90" t="n">
+      <c r="E70" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H57)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B70" s="2" t="n">
+    <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B71" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C70" s="90" t="n">
+      <c r="C71" s="91" t="n">
         <f aca="false">Auteur!B101</f>
         <v>1</v>
       </c>
-      <c r="D70" s="90" t="n">
+      <c r="D71" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G58)</f>
         <v>0</v>
       </c>
-      <c r="E70" s="90" t="n">
+      <c r="E71" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H58)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B71" s="2" t="n">
+    <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B72" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C71" s="90" t="n">
+      <c r="C72" s="91" t="n">
         <f aca="false">Auteur!B102</f>
         <v>2</v>
       </c>
-      <c r="D71" s="90" t="n">
+      <c r="D72" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G59)</f>
         <v>0</v>
       </c>
-      <c r="E71" s="90" t="n">
+      <c r="E72" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H59)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B72" s="2" t="n">
+    <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B73" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C72" s="90" t="n">
+      <c r="C73" s="91" t="n">
         <f aca="false">Auteur!B103</f>
         <v>3</v>
       </c>
-      <c r="D72" s="90" t="n">
+      <c r="D73" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G60)</f>
         <v>0</v>
       </c>
-      <c r="E72" s="90" t="n">
+      <c r="E73" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H60)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B73" s="2" t="n">
+    <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B74" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C73" s="90" t="n">
+      <c r="C74" s="91" t="n">
         <f aca="false">Auteur!B104</f>
         <v>4</v>
       </c>
-      <c r="D73" s="90" t="n">
+      <c r="D74" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G61)</f>
         <v>0</v>
       </c>
-      <c r="E73" s="90" t="n">
+      <c r="E74" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H61)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B74" s="2" t="n">
+    <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B75" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C74" s="90" t="n">
+      <c r="C75" s="91" t="n">
         <f aca="false">Auteur!B109</f>
         <v>1</v>
       </c>
-      <c r="D74" s="90" t="n">
+      <c r="D75" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G62)</f>
         <v>0</v>
       </c>
-      <c r="E74" s="90" t="n">
+      <c r="E75" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H62)</f>
         <v>0</v>
       </c>
-      <c r="IT74" s="90"/>
-    </row>
-    <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B75" s="2" t="n">
+      <c r="IT75" s="91"/>
+    </row>
+    <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B76" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C75" s="90" t="n">
+      <c r="C76" s="91" t="n">
         <f aca="false">Auteur!B110</f>
         <v>2</v>
       </c>
-      <c r="D75" s="90" t="n">
+      <c r="D76" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G63)</f>
         <v>0</v>
       </c>
-      <c r="E75" s="90" t="n">
+      <c r="E76" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H63)</f>
         <v>0</v>
       </c>
-      <c r="IT75" s="90"/>
-    </row>
-    <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B76" s="2" t="n">
+      <c r="IT76" s="91"/>
+    </row>
+    <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B77" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C76" s="90" t="n">
+      <c r="C77" s="91" t="n">
         <f aca="false">Auteur!B111</f>
         <v>3</v>
       </c>
-      <c r="D76" s="90" t="n">
+      <c r="D77" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G64)</f>
         <v>0</v>
       </c>
-      <c r="E76" s="90" t="n">
+      <c r="E77" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H64)</f>
         <v>0</v>
       </c>
-      <c r="IT76" s="90"/>
-    </row>
-    <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B77" s="2" t="n">
+      <c r="IT77" s="91"/>
+    </row>
+    <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B78" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C77" s="90" t="n">
+      <c r="C78" s="91" t="n">
         <f aca="false">Auteur!B112</f>
         <v>4</v>
       </c>
-      <c r="D77" s="90" t="n">
+      <c r="D78" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G65)</f>
         <v>0</v>
       </c>
-      <c r="E77" s="90" t="n">
+      <c r="E78" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H65)</f>
         <v>0</v>
       </c>
-      <c r="IT77" s="90"/>
-    </row>
-    <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B78" s="2" t="n">
+      <c r="IT78" s="91"/>
+    </row>
+    <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B79" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C78" s="90" t="n">
+      <c r="C79" s="91" t="n">
         <f aca="false">Auteur!B113</f>
         <v>5</v>
       </c>
-      <c r="D78" s="90" t="n">
+      <c r="D79" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G66)</f>
         <v>0</v>
       </c>
-      <c r="E78" s="90" t="n">
+      <c r="E79" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H66)</f>
         <v>0</v>
       </c>
-      <c r="IT78" s="90"/>
-    </row>
-    <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B79" s="2" t="n">
+      <c r="IT79" s="91"/>
+    </row>
+    <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B80" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C79" s="90" t="n">
+      <c r="C80" s="91" t="n">
         <f aca="false">Auteur!B118</f>
         <v>1</v>
       </c>
-      <c r="D79" s="90" t="n">
+      <c r="D80" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G67)</f>
         <v>0</v>
       </c>
-      <c r="E79" s="90" t="n">
+      <c r="E80" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H67)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B80" s="2" t="n">
+    <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B81" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C80" s="90" t="n">
+      <c r="C81" s="91" t="n">
         <f aca="false">Auteur!B119</f>
         <v>2</v>
       </c>
-      <c r="D80" s="90" t="n">
+      <c r="D81" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G68)</f>
         <v>0</v>
       </c>
-      <c r="E80" s="90" t="n">
+      <c r="E81" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H68)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B81" s="2" t="n">
+    <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B82" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C81" s="90" t="n">
+      <c r="C82" s="91" t="n">
         <f aca="false">Auteur!B120</f>
         <v>3</v>
       </c>
-      <c r="D81" s="90" t="n">
+      <c r="D82" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G69)</f>
         <v>0</v>
       </c>
-      <c r="E81" s="90" t="n">
+      <c r="E82" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H69)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B82" s="2" t="n">
+    <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B83" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C82" s="90" t="n">
+      <c r="C83" s="91" t="n">
         <f aca="false">Auteur!B121</f>
         <v>4</v>
       </c>
-      <c r="D82" s="90" t="n">
+      <c r="D83" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G70)</f>
         <v>0</v>
       </c>
-      <c r="E82" s="90" t="n">
+      <c r="E83" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H70)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B83" s="2" t="n">
+    <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B84" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="C83" s="90" t="n">
+      <c r="C84" s="91" t="n">
         <f aca="false">Auteur!B122</f>
         <v>5</v>
       </c>
-      <c r="D83" s="90" t="n">
+      <c r="D84" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G71)</f>
         <v>0</v>
       </c>
-      <c r="E83" s="90" t="n">
+      <c r="E84" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H71)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B84" s="2" t="n">
+    <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B85" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C84" s="90" t="s">
-        <v>80</v>
-      </c>
-      <c r="D84" s="90" t="str">
+      <c r="C85" s="91" t="s">
+        <v>83</v>
+      </c>
+      <c r="D85" s="91" t="str">
         <f aca="false">Auteur!C129</f>
         <v>Saisir question thème 1 ici</v>
       </c>
-      <c r="E84" s="90"/>
-    </row>
-    <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B85" s="2" t="n">
+      <c r="E85" s="91"/>
+    </row>
+    <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B86" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C85" s="90" t="n">
+      <c r="C86" s="91" t="n">
         <f aca="false">Auteur!B130</f>
         <v>1</v>
       </c>
-      <c r="D85" s="90" t="n">
+      <c r="D86" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G72)</f>
         <v>0</v>
       </c>
-      <c r="E85" s="90" t="n">
+      <c r="E86" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H72)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B86" s="2" t="n">
+    <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B87" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C86" s="90" t="n">
+      <c r="C87" s="91" t="n">
         <f aca="false">Auteur!B131</f>
         <v>2</v>
       </c>
-      <c r="D86" s="90" t="n">
+      <c r="D87" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G73)</f>
         <v>0</v>
       </c>
-      <c r="E86" s="90" t="n">
+      <c r="E87" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H73)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B87" s="2" t="n">
+    <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B88" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C87" s="90" t="n">
+      <c r="C88" s="91" t="n">
         <f aca="false">Auteur!B132</f>
         <v>3</v>
       </c>
-      <c r="D87" s="90" t="n">
+      <c r="D88" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G74)</f>
         <v>0</v>
       </c>
-      <c r="E87" s="90" t="n">
+      <c r="E88" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H74)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B88" s="2" t="n">
+    <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B89" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C88" s="90" t="n">
+      <c r="C89" s="91" t="n">
         <f aca="false">Auteur!B133</f>
         <v>4</v>
       </c>
-      <c r="D88" s="90" t="n">
+      <c r="D89" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G75)</f>
         <v>0</v>
       </c>
-      <c r="E88" s="90" t="n">
+      <c r="E89" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H75)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B89" s="2" t="n">
+    <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B90" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C89" s="90" t="s">
-        <v>81</v>
-      </c>
-      <c r="D89" s="90" t="str">
+      <c r="C90" s="91" t="s">
+        <v>84</v>
+      </c>
+      <c r="D90" s="91" t="str">
         <f aca="false">Auteur!C140</f>
         <v>Saisir question thème 2 ici</v>
       </c>
-      <c r="E89" s="90"/>
-    </row>
-    <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B90" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="C90" s="90" t="n">
-        <v>5</v>
-      </c>
-      <c r="D90" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!G76)</f>
-        <v>0</v>
-      </c>
-      <c r="E90" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!H76)</f>
-        <v>0</v>
-      </c>
+      <c r="E90" s="91"/>
     </row>
     <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="n">
@@ -5933,15 +6107,15 @@
       <c r="B91" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C91" s="90" t="n">
-        <v>6</v>
-      </c>
-      <c r="D91" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!G77)</f>
-        <v>0</v>
-      </c>
-      <c r="E91" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!H77)</f>
+      <c r="C91" s="91" t="n">
+        <v>5</v>
+      </c>
+      <c r="D91" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G76)</f>
+        <v>0</v>
+      </c>
+      <c r="E91" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H76)</f>
         <v>0</v>
       </c>
     </row>
@@ -5953,15 +6127,15 @@
       <c r="B92" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C92" s="90" t="n">
-        <v>7</v>
-      </c>
-      <c r="D92" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!G78)</f>
-        <v>0</v>
-      </c>
-      <c r="E92" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!H78)</f>
+      <c r="C92" s="91" t="n">
+        <v>6</v>
+      </c>
+      <c r="D92" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G77)</f>
+        <v>0</v>
+      </c>
+      <c r="E92" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H77)</f>
         <v>0</v>
       </c>
     </row>
@@ -5973,15 +6147,15 @@
       <c r="B93" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="C93" s="90" t="n">
-        <v>8</v>
-      </c>
-      <c r="D93" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!G79)</f>
-        <v>0</v>
-      </c>
-      <c r="E93" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!H79)</f>
+      <c r="C93" s="91" t="n">
+        <v>7</v>
+      </c>
+      <c r="D93" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G78)</f>
+        <v>0</v>
+      </c>
+      <c r="E93" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H78)</f>
         <v>0</v>
       </c>
     </row>
@@ -5991,20 +6165,19 @@
         <v>0</v>
       </c>
       <c r="B94" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="C94" s="90" t="n">
-        <v>1</v>
-      </c>
-      <c r="D94" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!G80)</f>
-        <v>0</v>
-      </c>
-      <c r="E94" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!H80)</f>
-        <v>0</v>
-      </c>
-      <c r="IT94" s="90"/>
+        <v>13</v>
+      </c>
+      <c r="C94" s="91" t="n">
+        <v>8</v>
+      </c>
+      <c r="D94" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G79)</f>
+        <v>0</v>
+      </c>
+      <c r="E94" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H79)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="n">
@@ -6014,18 +6187,18 @@
       <c r="B95" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C95" s="90" t="n">
-        <v>2</v>
-      </c>
-      <c r="D95" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!G81)</f>
-        <v>0</v>
-      </c>
-      <c r="E95" s="90" t="n">
-        <f aca="true">INDIRECT(Adresses!H81)</f>
-        <v>0</v>
-      </c>
-      <c r="IT95" s="90"/>
+      <c r="C95" s="91" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G80)</f>
+        <v>0</v>
+      </c>
+      <c r="E95" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H80)</f>
+        <v>0</v>
+      </c>
+      <c r="IT95" s="91"/>
     </row>
     <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="n">
@@ -6035,213 +6208,213 @@
       <c r="B96" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C96" s="90" t="n">
+      <c r="C96" s="91" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G81)</f>
+        <v>0</v>
+      </c>
+      <c r="E96" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H81)</f>
+        <v>0</v>
+      </c>
+      <c r="IT96" s="91"/>
+    </row>
+    <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C97" s="91" t="n">
         <f aca="false">Auteur!B155</f>
         <v>3</v>
       </c>
-      <c r="D96" s="90" t="n">
+      <c r="D97" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G82)</f>
         <v>0</v>
       </c>
-      <c r="E96" s="90" t="n">
+      <c r="E97" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H82)</f>
         <v>0</v>
       </c>
-      <c r="IT96" s="90"/>
-    </row>
-    <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B97" s="2" t="n">
+      <c r="IT97" s="91"/>
+    </row>
+    <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B98" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C97" s="90" t="n">
+      <c r="C98" s="91" t="n">
         <f aca="false">Auteur!B156</f>
         <v>4</v>
       </c>
-      <c r="D97" s="90" t="n">
+      <c r="D98" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G83)</f>
         <v>0</v>
       </c>
-      <c r="E97" s="90" t="n">
+      <c r="E98" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H83)</f>
         <v>0</v>
       </c>
-      <c r="IT97" s="90"/>
-    </row>
-    <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B98" s="2" t="n">
+      <c r="IT98" s="91"/>
+    </row>
+    <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B99" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C98" s="90" t="n">
+      <c r="C99" s="91" t="n">
         <f aca="false">Auteur!B157</f>
         <v>5</v>
       </c>
-      <c r="D98" s="90" t="n">
+      <c r="D99" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G84)</f>
         <v>0</v>
       </c>
-      <c r="E98" s="90" t="n">
+      <c r="E99" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H84)</f>
         <v>0</v>
       </c>
-      <c r="IT98" s="91"/>
-    </row>
-    <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B99" s="2" t="n">
+      <c r="IT99" s="92"/>
+    </row>
+    <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B100" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C99" s="90" t="n">
+      <c r="C100" s="91" t="n">
         <f aca="false">Auteur!B158</f>
         <v>6</v>
       </c>
-      <c r="D99" s="90" t="n">
+      <c r="D100" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G85)</f>
         <v>0</v>
       </c>
-      <c r="E99" s="90" t="n">
+      <c r="E100" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H85)</f>
         <v>0</v>
       </c>
-      <c r="IT99" s="91"/>
-    </row>
-    <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B100" s="2" t="n">
+      <c r="IT100" s="92"/>
+    </row>
+    <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B101" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C100" s="90" t="n">
+      <c r="C101" s="91" t="n">
         <f aca="false">Auteur!B159</f>
         <v>7</v>
       </c>
-      <c r="D100" s="90" t="n">
+      <c r="D101" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G86)</f>
         <v>0</v>
       </c>
-      <c r="E100" s="90" t="n">
+      <c r="E101" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H86)</f>
         <v>0</v>
       </c>
-      <c r="IT100" s="91"/>
-    </row>
-    <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B101" s="2" t="n">
+      <c r="IT101" s="92"/>
+    </row>
+    <row r="102" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B102" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C101" s="90" t="n">
+      <c r="C102" s="91" t="n">
         <f aca="false">Auteur!B160</f>
         <v>8</v>
       </c>
-      <c r="D101" s="90" t="n">
+      <c r="D102" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G87)</f>
         <v>0</v>
       </c>
-      <c r="E101" s="90" t="n">
+      <c r="E102" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H87)</f>
         <v>0</v>
       </c>
-      <c r="IT101" s="91"/>
-    </row>
-    <row r="102" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B102" s="2" t="n">
+      <c r="IT102" s="92"/>
+    </row>
+    <row r="103" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B103" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C102" s="90" t="n">
+      <c r="C103" s="91" t="n">
         <f aca="false">Auteur!B161</f>
         <v>9</v>
       </c>
-      <c r="D102" s="90" t="n">
+      <c r="D103" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G88)</f>
         <v>0</v>
       </c>
-      <c r="E102" s="90" t="n">
+      <c r="E103" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H88)</f>
         <v>0</v>
       </c>
-      <c r="IT102" s="91"/>
-    </row>
-    <row r="103" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B103" s="2" t="n">
+      <c r="IT103" s="92"/>
+    </row>
+    <row r="104" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B104" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C103" s="90" t="n">
+      <c r="C104" s="91" t="n">
         <f aca="false">Auteur!B162</f>
         <v>10</v>
       </c>
-      <c r="D103" s="90" t="n">
+      <c r="D104" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G89)</f>
         <v>0</v>
       </c>
-      <c r="E103" s="90" t="n">
+      <c r="E104" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H89)</f>
         <v>0</v>
       </c>
-      <c r="IT103" s="91"/>
-    </row>
-    <row r="104" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B104" s="2" t="n">
+      <c r="IT104" s="92"/>
+    </row>
+    <row r="105" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B105" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C104" s="90" t="n">
+      <c r="C105" s="91" t="n">
         <f aca="false">Auteur!B167</f>
         <v>1</v>
       </c>
-      <c r="D104" s="90" t="n">
+      <c r="D105" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!G90)</f>
         <v>0</v>
       </c>
-      <c r="E104" s="90" t="n">
+      <c r="E105" s="91" t="n">
         <f aca="true">INDIRECT(Adresses!H90)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="2" t="n">
-        <f aca="false">Auteur!$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="B105" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C105" s="90" t="n">
-        <f aca="false">C104+1</f>
-        <v>2</v>
-      </c>
-      <c r="D105" s="90" t="n">
-        <f aca="false">$D$104</f>
-        <v>0</v>
-      </c>
-      <c r="E105" s="90" t="n">
-        <f aca="false">E104</f>
         <v>0</v>
       </c>
     </row>
@@ -6253,15 +6426,15 @@
       <c r="B106" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C106" s="90" t="n">
+      <c r="C106" s="91" t="n">
         <f aca="false">C105+1</f>
-        <v>3</v>
-      </c>
-      <c r="D106" s="90" t="n">
-        <f aca="false">$D$104</f>
-        <v>0</v>
-      </c>
-      <c r="E106" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D106" s="91" t="n">
+        <f aca="false">$D$105</f>
+        <v>0</v>
+      </c>
+      <c r="E106" s="91" t="n">
         <f aca="false">E105</f>
         <v>0</v>
       </c>
@@ -6274,15 +6447,15 @@
       <c r="B107" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C107" s="90" t="n">
+      <c r="C107" s="91" t="n">
         <f aca="false">C106+1</f>
-        <v>4</v>
-      </c>
-      <c r="D107" s="90" t="n">
-        <f aca="false">$D$104</f>
-        <v>0</v>
-      </c>
-      <c r="E107" s="90" t="n">
+        <v>3</v>
+      </c>
+      <c r="D107" s="91" t="n">
+        <f aca="false">$D$105</f>
+        <v>0</v>
+      </c>
+      <c r="E107" s="91" t="n">
         <f aca="false">E106</f>
         <v>0</v>
       </c>
@@ -6295,15 +6468,15 @@
       <c r="B108" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C108" s="90" t="n">
+      <c r="C108" s="91" t="n">
         <f aca="false">C107+1</f>
-        <v>5</v>
-      </c>
-      <c r="D108" s="90" t="n">
-        <f aca="false">$D$104</f>
-        <v>0</v>
-      </c>
-      <c r="E108" s="90" t="n">
+        <v>4</v>
+      </c>
+      <c r="D108" s="91" t="n">
+        <f aca="false">$D$105</f>
+        <v>0</v>
+      </c>
+      <c r="E108" s="91" t="n">
         <f aca="false">E107</f>
         <v>0</v>
       </c>
@@ -6316,15 +6489,15 @@
       <c r="B109" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C109" s="90" t="n">
+      <c r="C109" s="91" t="n">
         <f aca="false">C108+1</f>
-        <v>6</v>
-      </c>
-      <c r="D109" s="90" t="n">
-        <f aca="false">$D$104</f>
-        <v>0</v>
-      </c>
-      <c r="E109" s="90" t="n">
+        <v>5</v>
+      </c>
+      <c r="D109" s="91" t="n">
+        <f aca="false">$D$105</f>
+        <v>0</v>
+      </c>
+      <c r="E109" s="91" t="n">
         <f aca="false">E108</f>
         <v>0</v>
       </c>
@@ -6337,15 +6510,15 @@
       <c r="B110" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C110" s="90" t="n">
+      <c r="C110" s="91" t="n">
         <f aca="false">C109+1</f>
-        <v>7</v>
-      </c>
-      <c r="D110" s="90" t="n">
-        <f aca="false">$D$104</f>
-        <v>0</v>
-      </c>
-      <c r="E110" s="90" t="n">
+        <v>6</v>
+      </c>
+      <c r="D110" s="91" t="n">
+        <f aca="false">$D$105</f>
+        <v>0</v>
+      </c>
+      <c r="E110" s="91" t="n">
         <f aca="false">E109</f>
         <v>0</v>
       </c>
@@ -6358,16 +6531,184 @@
       <c r="B111" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C111" s="90" t="n">
+      <c r="C111" s="91" t="n">
         <f aca="false">C110+1</f>
+        <v>7</v>
+      </c>
+      <c r="D111" s="91" t="n">
+        <f aca="false">$D$105</f>
+        <v>0</v>
+      </c>
+      <c r="E111" s="91" t="n">
+        <f aca="false">E110</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B112" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C112" s="91" t="n">
+        <f aca="false">C111+1</f>
         <v>8</v>
       </c>
-      <c r="D111" s="90" t="n">
-        <f aca="false">$D$104</f>
-        <v>0</v>
-      </c>
-      <c r="E111" s="90" t="n">
-        <f aca="false">E110</f>
+      <c r="D112" s="91" t="n">
+        <f aca="false">$D$105</f>
+        <v>0</v>
+      </c>
+      <c r="E112" s="91" t="n">
+        <f aca="false">E111</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B113" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C113" s="91" t="n">
+        <f aca="false">Auteur!B172</f>
+        <v>1</v>
+      </c>
+      <c r="D113" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G91)</f>
+        <v>0</v>
+      </c>
+      <c r="E113" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H91)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B114" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C114" s="91" t="n">
+        <f aca="false">Auteur!B173</f>
+        <v>2</v>
+      </c>
+      <c r="D114" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G92)</f>
+        <v>0</v>
+      </c>
+      <c r="E114" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H92)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B115" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C115" s="91" t="n">
+        <f aca="false">Auteur!B174</f>
+        <v>3</v>
+      </c>
+      <c r="D115" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G93)</f>
+        <v>0</v>
+      </c>
+      <c r="E115" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H93)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B116" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C116" s="91" t="n">
+        <f aca="false">Auteur!B175</f>
+        <v>4</v>
+      </c>
+      <c r="D116" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G94)</f>
+        <v>0</v>
+      </c>
+      <c r="E116" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H94)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B117" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C117" s="91" t="n">
+        <f aca="false">Auteur!B176</f>
+        <v>5</v>
+      </c>
+      <c r="D117" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G95)</f>
+        <v>0</v>
+      </c>
+      <c r="E117" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H95)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B118" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C118" s="91" t="n">
+        <f aca="false">Auteur!B177</f>
+        <v>6</v>
+      </c>
+      <c r="D118" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G96)</f>
+        <v>0</v>
+      </c>
+      <c r="E118" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H96)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2" t="n">
+        <f aca="false">Auteur!$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="B119" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C119" s="91" t="n">
+        <f aca="false">Auteur!B178</f>
+        <v>7</v>
+      </c>
+      <c r="D119" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!G97)</f>
+        <v>0</v>
+      </c>
+      <c r="E119" s="91" t="n">
+        <f aca="true">INDIRECT(Adresses!H97)</f>
         <v>0</v>
       </c>
     </row>
@@ -6397,77 +6738,77 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="92"/>
-      <c r="C2" s="93" t="n">
+      <c r="B2" s="93"/>
+      <c r="C2" s="94" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="93"/>
+      <c r="D2" s="94"/>
       <c r="G2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="94" t="s">
+      <c r="A3" s="95" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="94"/>
-      <c r="C3" s="95" t="s">
-        <v>82</v>
-      </c>
-      <c r="D3" s="95"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="96" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="96"/>
       <c r="G3" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="94" t="s">
+      <c r="A4" s="95" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="94"/>
-      <c r="C4" s="95" t="s">
-        <v>84</v>
-      </c>
-      <c r="D4" s="95"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="96" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="96"/>
       <c r="G4" s="2" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="94" t="s">
+      <c r="A5" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="95" t="s">
-        <v>85</v>
-      </c>
-      <c r="D5" s="95"/>
+      <c r="B5" s="95"/>
+      <c r="C5" s="96" t="s">
+        <v>88</v>
+      </c>
+      <c r="D5" s="96"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="94" t="s">
-        <v>86</v>
-      </c>
-      <c r="B6" s="94"/>
-      <c r="C6" s="95"/>
-      <c r="D6" s="95"/>
+      <c r="A6" s="95" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="95"/>
+      <c r="C6" s="96"/>
+      <c r="D6" s="96"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="94" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="94"/>
-      <c r="C7" s="95"/>
-      <c r="D7" s="95"/>
+      <c r="A7" s="95" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="95"/>
+      <c r="C7" s="96"/>
+      <c r="D7" s="96"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="96" t="s">
-        <v>88</v>
-      </c>
-      <c r="B8" s="96"/>
-      <c r="C8" s="97"/>
-      <c r="D8" s="97"/>
+      <c r="A8" s="97" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" s="97"/>
+      <c r="C8" s="98"/>
+      <c r="D8" s="98"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10"/>
@@ -6476,165 +6817,165 @@
       <c r="D9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="98" t="s">
-        <v>89</v>
-      </c>
-      <c r="B10" s="98"/>
-      <c r="C10" s="98"/>
-      <c r="D10" s="98"/>
+      <c r="A10" s="99" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="99"/>
+      <c r="C10" s="99"/>
+      <c r="D10" s="99"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="99"/>
-      <c r="B11" s="99"/>
-      <c r="C11" s="99"/>
-      <c r="D11" s="99"/>
+      <c r="A11" s="100"/>
+      <c r="B11" s="100"/>
+      <c r="C11" s="100"/>
+      <c r="D11" s="100"/>
     </row>
     <row r="12" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="100" t="s">
-        <v>90</v>
-      </c>
-      <c r="B12" s="100"/>
-      <c r="C12" s="100" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="101"/>
+      <c r="A12" s="101" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="101"/>
+      <c r="C12" s="101" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="102"/>
     </row>
     <row r="13" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="102" t="s">
+      <c r="A13" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="102"/>
-      <c r="C13" s="103" t="s">
-        <v>91</v>
-      </c>
-      <c r="D13" s="104" t="s">
-        <v>92</v>
+      <c r="B13" s="103"/>
+      <c r="C13" s="104" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13" s="105" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="105" t="s">
+      <c r="A14" s="106" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="105"/>
-      <c r="C14" s="105"/>
-      <c r="D14" s="105"/>
+      <c r="B14" s="106"/>
+      <c r="C14" s="106"/>
+      <c r="D14" s="106"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="105"/>
-      <c r="B15" s="105"/>
-      <c r="C15" s="105"/>
-      <c r="D15" s="105"/>
+      <c r="A15" s="106"/>
+      <c r="B15" s="106"/>
+      <c r="C15" s="106"/>
+      <c r="D15" s="106"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="105"/>
-      <c r="B16" s="105"/>
-      <c r="C16" s="105"/>
-      <c r="D16" s="105"/>
+      <c r="A16" s="106"/>
+      <c r="B16" s="106"/>
+      <c r="C16" s="106"/>
+      <c r="D16" s="106"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="106" t="n">
+      <c r="A17" s="107" t="n">
         <v>1</v>
       </c>
-      <c r="B17" s="107" t="n">
-        <f aca="false">'Vers BD'!D22</f>
-        <v>0</v>
-      </c>
-      <c r="C17" s="107"/>
-      <c r="D17" s="108" t="n">
-        <f aca="false">'Vers BD'!E22</f>
+      <c r="B17" s="108" t="n">
+        <f aca="false">'Vers BD'!D23</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="108"/>
+      <c r="D17" s="109" t="n">
+        <f aca="false">'Vers BD'!E23</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="106" t="n">
+      <c r="A18" s="107" t="n">
         <v>2</v>
       </c>
-      <c r="B18" s="107" t="s">
-        <v>93</v>
-      </c>
-      <c r="C18" s="107"/>
-      <c r="D18" s="108" t="s">
-        <v>94</v>
+      <c r="B18" s="108" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" s="108"/>
+      <c r="D18" s="109" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="106" t="n">
+      <c r="A19" s="107" t="n">
         <v>3</v>
       </c>
-      <c r="B19" s="107" t="s">
-        <v>95</v>
-      </c>
-      <c r="C19" s="107"/>
-      <c r="D19" s="108" t="s">
-        <v>96</v>
+      <c r="B19" s="108" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" s="108"/>
+      <c r="D19" s="109" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="106" t="n">
+      <c r="A20" s="107" t="n">
         <v>4</v>
       </c>
-      <c r="B20" s="107" t="s">
-        <v>97</v>
-      </c>
-      <c r="C20" s="107"/>
-      <c r="D20" s="108" t="s">
-        <v>98</v>
+      <c r="B20" s="108" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="108"/>
+      <c r="D20" s="109" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="105" t="s">
+      <c r="A21" s="106" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="105"/>
-      <c r="C21" s="105"/>
-      <c r="D21" s="105"/>
+      <c r="B21" s="106"/>
+      <c r="C21" s="106"/>
+      <c r="D21" s="106"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="106" t="n">
+      <c r="A22" s="107" t="n">
         <v>1</v>
       </c>
-      <c r="B22" s="107" t="s">
-        <v>99</v>
-      </c>
-      <c r="C22" s="107"/>
-      <c r="D22" s="108" t="s">
-        <v>100</v>
+      <c r="B22" s="108" t="s">
+        <v>102</v>
+      </c>
+      <c r="C22" s="108"/>
+      <c r="D22" s="109" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="106" t="n">
+      <c r="A23" s="107" t="n">
         <v>2</v>
       </c>
-      <c r="B23" s="107" t="s">
-        <v>101</v>
-      </c>
-      <c r="C23" s="107"/>
-      <c r="D23" s="108" t="s">
-        <v>102</v>
+      <c r="B23" s="108" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="108"/>
+      <c r="D23" s="109" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="106" t="n">
+      <c r="A24" s="107" t="n">
         <v>3</v>
       </c>
-      <c r="B24" s="107" t="s">
-        <v>103</v>
-      </c>
-      <c r="C24" s="107"/>
-      <c r="D24" s="108" t="s">
-        <v>104</v>
+      <c r="B24" s="108" t="s">
+        <v>106</v>
+      </c>
+      <c r="C24" s="108"/>
+      <c r="D24" s="109" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="106" t="n">
+      <c r="A25" s="107" t="n">
         <v>4</v>
       </c>
-      <c r="B25" s="107" t="s">
-        <v>105</v>
-      </c>
-      <c r="C25" s="107"/>
-      <c r="D25" s="108" t="s">
-        <v>106</v>
+      <c r="B25" s="108" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" s="108"/>
+      <c r="D25" s="109" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6644,97 +6985,97 @@
       <c r="D26" s="28"/>
     </row>
     <row r="27" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="98" t="s">
-        <v>107</v>
-      </c>
-      <c r="B27" s="98"/>
-      <c r="C27" s="98"/>
-      <c r="D27" s="98"/>
+      <c r="A27" s="99" t="s">
+        <v>110</v>
+      </c>
+      <c r="B27" s="99"/>
+      <c r="C27" s="99"/>
+      <c r="D27" s="99"/>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="99"/>
-      <c r="B28" s="99"/>
-      <c r="C28" s="99"/>
-      <c r="D28" s="99"/>
+      <c r="A28" s="100"/>
+      <c r="B28" s="100"/>
+      <c r="C28" s="100"/>
+      <c r="D28" s="100"/>
     </row>
     <row r="29" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="100" t="s">
-        <v>108</v>
-      </c>
-      <c r="B29" s="100"/>
-      <c r="C29" s="109" t="s">
-        <v>74</v>
-      </c>
-      <c r="D29" s="110" t="s">
-        <v>109</v>
+      <c r="A29" s="101" t="s">
+        <v>111</v>
+      </c>
+      <c r="B29" s="101"/>
+      <c r="C29" s="110" t="s">
+        <v>77</v>
+      </c>
+      <c r="D29" s="111" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="111" t="s">
-        <v>110</v>
-      </c>
-      <c r="B30" s="111"/>
-      <c r="C30" s="109"/>
-      <c r="D30" s="110"/>
+      <c r="A30" s="112" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="112"/>
+      <c r="C30" s="110"/>
+      <c r="D30" s="111"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="106" t="n">
+      <c r="A31" s="107" t="n">
         <v>1</v>
       </c>
-      <c r="B31" s="107" t="s">
-        <v>111</v>
-      </c>
-      <c r="C31" s="107"/>
-      <c r="D31" s="108" t="s">
-        <v>112</v>
+      <c r="B31" s="108" t="s">
+        <v>114</v>
+      </c>
+      <c r="C31" s="108"/>
+      <c r="D31" s="109" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="106" t="n">
+      <c r="A32" s="107" t="n">
         <v>2</v>
       </c>
-      <c r="B32" s="107" t="s">
-        <v>113</v>
-      </c>
-      <c r="C32" s="107"/>
-      <c r="D32" s="108" t="s">
-        <v>114</v>
+      <c r="B32" s="108" t="s">
+        <v>116</v>
+      </c>
+      <c r="C32" s="108"/>
+      <c r="D32" s="109" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="106" t="n">
+      <c r="A33" s="107" t="n">
         <v>3</v>
       </c>
-      <c r="B33" s="107" t="s">
-        <v>115</v>
-      </c>
-      <c r="C33" s="107"/>
-      <c r="D33" s="108" t="s">
-        <v>116</v>
+      <c r="B33" s="108" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" s="108"/>
+      <c r="D33" s="109" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="106" t="n">
+      <c r="A34" s="107" t="n">
         <v>4</v>
       </c>
-      <c r="B34" s="107" t="s">
-        <v>117</v>
-      </c>
-      <c r="C34" s="107"/>
-      <c r="D34" s="108" t="s">
-        <v>118</v>
+      <c r="B34" s="108" t="s">
+        <v>120</v>
+      </c>
+      <c r="C34" s="108"/>
+      <c r="D34" s="109" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="106" t="n">
+      <c r="A35" s="107" t="n">
         <v>5</v>
       </c>
-      <c r="B35" s="107" t="s">
-        <v>119</v>
-      </c>
-      <c r="C35" s="107"/>
-      <c r="D35" s="108" t="s">
-        <v>120</v>
+      <c r="B35" s="108" t="s">
+        <v>122</v>
+      </c>
+      <c r="C35" s="108"/>
+      <c r="D35" s="109" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6744,92 +7085,92 @@
       <c r="D36" s="34"/>
     </row>
     <row r="37" customFormat="false" ht="17.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="100" t="s">
-        <v>121</v>
-      </c>
-      <c r="B37" s="100"/>
-      <c r="C37" s="109" t="s">
-        <v>74</v>
-      </c>
-      <c r="D37" s="110" t="s">
-        <v>122</v>
+      <c r="A37" s="101" t="s">
+        <v>124</v>
+      </c>
+      <c r="B37" s="101"/>
+      <c r="C37" s="110" t="s">
+        <v>77</v>
+      </c>
+      <c r="D37" s="111" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="111" t="s">
-        <v>110</v>
-      </c>
-      <c r="B38" s="111"/>
-      <c r="C38" s="109"/>
-      <c r="D38" s="110"/>
+      <c r="A38" s="112" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38" s="112"/>
+      <c r="C38" s="110"/>
+      <c r="D38" s="111"/>
     </row>
     <row r="39" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="106" t="n">
+      <c r="A39" s="107" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="107" t="s">
-        <v>123</v>
-      </c>
-      <c r="C39" s="107"/>
-      <c r="D39" s="108" t="s">
-        <v>124</v>
+      <c r="B39" s="108" t="s">
+        <v>126</v>
+      </c>
+      <c r="C39" s="108"/>
+      <c r="D39" s="109" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="106" t="n">
+      <c r="A40" s="107" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="107" t="s">
-        <v>125</v>
-      </c>
-      <c r="C40" s="107"/>
-      <c r="D40" s="108" t="s">
-        <v>126</v>
+      <c r="B40" s="108" t="s">
+        <v>128</v>
+      </c>
+      <c r="C40" s="108"/>
+      <c r="D40" s="109" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="106" t="n">
+      <c r="A41" s="107" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="107" t="s">
-        <v>127</v>
-      </c>
-      <c r="C41" s="107"/>
-      <c r="D41" s="108" t="s">
-        <v>128</v>
+      <c r="B41" s="108" t="s">
+        <v>130</v>
+      </c>
+      <c r="C41" s="108"/>
+      <c r="D41" s="109" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="106" t="n">
+      <c r="A42" s="107" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="107" t="s">
-        <v>129</v>
-      </c>
-      <c r="C42" s="107"/>
-      <c r="D42" s="108" t="s">
-        <v>130</v>
+      <c r="B42" s="108" t="s">
+        <v>132</v>
+      </c>
+      <c r="C42" s="108"/>
+      <c r="D42" s="109" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="107" t="n">
+      <c r="A43" s="108" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="112" t="s">
-        <v>131</v>
-      </c>
-      <c r="C43" s="112"/>
-      <c r="D43" s="113" t="s">
-        <v>132</v>
+      <c r="B43" s="113" t="s">
+        <v>134</v>
+      </c>
+      <c r="C43" s="113"/>
+      <c r="D43" s="114" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="77.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="107"/>
-      <c r="B44" s="106" t="s">
-        <v>133</v>
-      </c>
-      <c r="C44" s="106"/>
-      <c r="D44" s="113"/>
+      <c r="A44" s="108"/>
+      <c r="B44" s="107" t="s">
+        <v>136</v>
+      </c>
+      <c r="C44" s="107"/>
+      <c r="D44" s="114"/>
     </row>
   </sheetData>
   <mergeCells count="54">
@@ -6917,21 +7258,21 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="114" t="s">
-        <v>134</v>
+      <c r="A1" s="115" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>59</v>
@@ -6939,7 +7280,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>59</v>
@@ -6947,7 +7288,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>58</v>
@@ -6955,36 +7296,36 @@
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="115" t="s">
-        <v>141</v>
-      </c>
-      <c r="B8" s="116" t="s">
-        <v>142</v>
-      </c>
-      <c r="C8" s="116" t="s">
-        <v>143</v>
-      </c>
-      <c r="D8" s="116" t="s">
+      <c r="A8" s="116" t="s">
         <v>144</v>
       </c>
-      <c r="E8" s="116" t="s">
+      <c r="B8" s="117" t="s">
         <v>145</v>
       </c>
-      <c r="F8" s="116" t="s">
+      <c r="C8" s="117" t="s">
         <v>146</v>
       </c>
-      <c r="G8" s="116" t="s">
+      <c r="D8" s="117" t="s">
         <v>147</v>
       </c>
-      <c r="H8" s="116" t="s">
+      <c r="E8" s="117" t="s">
         <v>148</v>
+      </c>
+      <c r="F8" s="117" t="s">
+        <v>149</v>
+      </c>
+      <c r="G8" s="117" t="s">
+        <v>150</v>
+      </c>
+      <c r="H8" s="117" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7006,7 +7347,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D9</f>
         <v>Auteur!D11</v>
       </c>
-      <c r="F9" s="114" t="n">
+      <c r="F9" s="115" t="n">
         <v>14</v>
       </c>
       <c r="G9" s="2" t="str">
@@ -7156,7 +7497,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D17</f>
         <v>Auteur!D25</v>
       </c>
-      <c r="F17" s="114" t="n">
+      <c r="F17" s="115" t="n">
         <v>27</v>
       </c>
       <c r="G17" s="2" t="str">
@@ -7256,7 +7597,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D22</f>
         <v>Auteur!D34</v>
       </c>
-      <c r="F22" s="114" t="n">
+      <c r="F22" s="115" t="n">
         <v>36</v>
       </c>
       <c r="G22" s="2" t="str">
@@ -7356,7 +7697,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D27</f>
         <v>Auteur!D43</v>
       </c>
-      <c r="F27" s="114" t="n">
+      <c r="F27" s="115" t="n">
         <v>45</v>
       </c>
       <c r="G27" s="2" t="str">
@@ -7456,7 +7797,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D32</f>
         <v>Auteur!D52</v>
       </c>
-      <c r="F32" s="114" t="n">
+      <c r="F32" s="115" t="n">
         <v>54</v>
       </c>
       <c r="G32" s="2" t="str">
@@ -7556,7 +7897,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D37</f>
         <v>Auteur!D61</v>
       </c>
-      <c r="F37" s="114" t="n">
+      <c r="F37" s="115" t="n">
         <v>64</v>
       </c>
       <c r="G37" s="2" t="str">
@@ -7623,7 +7964,7 @@
       <c r="A41" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F41" s="114" t="n">
+      <c r="F41" s="115" t="n">
         <v>68</v>
       </c>
       <c r="G41" s="2" t="str">
@@ -7706,7 +8047,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D45</f>
         <v>Auteur!D74</v>
       </c>
-      <c r="F45" s="114" t="n">
+      <c r="F45" s="115" t="n">
         <v>76</v>
       </c>
       <c r="G45" s="2" t="str">
@@ -7806,7 +8147,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D50</f>
         <v>Auteur!D83</v>
       </c>
-      <c r="F50" s="114" t="n">
+      <c r="F50" s="115" t="n">
         <v>85</v>
       </c>
       <c r="G50" s="2" t="str">
@@ -7906,7 +8247,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D55</f>
         <v>Auteur!D92</v>
       </c>
-      <c r="F55" s="114" t="n">
+      <c r="F55" s="115" t="n">
         <v>94</v>
       </c>
       <c r="G55" s="2" t="str">
@@ -7972,7 +8313,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D58</f>
         <v>Auteur!D99</v>
       </c>
-      <c r="F58" s="114" t="n">
+      <c r="F58" s="115" t="n">
         <v>101</v>
       </c>
       <c r="G58" s="2" t="str">
@@ -8055,7 +8396,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D62</f>
         <v>Auteur!D107</v>
       </c>
-      <c r="F62" s="114" t="n">
+      <c r="F62" s="115" t="n">
         <v>109</v>
       </c>
       <c r="G62" s="2" t="str">
@@ -8158,7 +8499,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D67</f>
         <v>Auteur!D116</v>
       </c>
-      <c r="F67" s="114" t="n">
+      <c r="F67" s="115" t="n">
         <v>118</v>
       </c>
       <c r="G67" s="2" t="str">
@@ -8240,41 +8581,41 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="117" t="n">
+      <c r="A72" s="118" t="n">
         <v>13</v>
       </c>
-      <c r="B72" s="118" t="n">
+      <c r="B72" s="119" t="n">
         <v>124</v>
       </c>
-      <c r="C72" s="118" t="str">
+      <c r="C72" s="119" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;B72</f>
         <v>Auteur!D124</v>
       </c>
-      <c r="D72" s="118" t="n">
+      <c r="D72" s="119" t="n">
         <v>125</v>
       </c>
-      <c r="E72" s="118" t="str">
+      <c r="E72" s="119" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D72</f>
         <v>Auteur!D125</v>
       </c>
-      <c r="F72" s="119" t="n">
+      <c r="F72" s="120" t="n">
         <v>130</v>
       </c>
-      <c r="G72" s="118" t="str">
+      <c r="G72" s="119" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F72</f>
         <v>Auteur!C130</v>
       </c>
-      <c r="H72" s="120" t="str">
+      <c r="H72" s="121" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F72</f>
         <v>Auteur!D130</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="121" t="n">
+      <c r="A73" s="122" t="n">
         <f aca="false">A69+1</f>
         <v>13</v>
       </c>
-      <c r="F73" s="122" t="n">
+      <c r="F73" s="123" t="n">
         <f aca="false">F72+1</f>
         <v>131</v>
       </c>
@@ -8282,16 +8623,16 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F73</f>
         <v>Auteur!C131</v>
       </c>
-      <c r="H73" s="123" t="str">
+      <c r="H73" s="124" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F73</f>
         <v>Auteur!D131</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="121" t="n">
+      <c r="A74" s="122" t="n">
         <v>13</v>
       </c>
-      <c r="F74" s="122" t="n">
+      <c r="F74" s="123" t="n">
         <f aca="false">F73+1</f>
         <v>132</v>
       </c>
@@ -8299,16 +8640,16 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F74</f>
         <v>Auteur!C132</v>
       </c>
-      <c r="H74" s="123" t="str">
+      <c r="H74" s="124" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F74</f>
         <v>Auteur!D132</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="121" t="n">
+      <c r="A75" s="122" t="n">
         <v>13</v>
       </c>
-      <c r="F75" s="122" t="n">
+      <c r="F75" s="123" t="n">
         <f aca="false">F74+1</f>
         <v>133</v>
       </c>
@@ -8316,75 +8657,75 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F75</f>
         <v>Auteur!C133</v>
       </c>
-      <c r="H75" s="123" t="str">
+      <c r="H75" s="124" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F75</f>
         <v>Auteur!D133</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="121" t="n">
+      <c r="A76" s="122" t="n">
         <v>13</v>
       </c>
-      <c r="F76" s="122" t="n">
+      <c r="F76" s="123" t="n">
         <v>141</v>
       </c>
       <c r="G76" s="2" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F76</f>
         <v>Auteur!C141</v>
       </c>
-      <c r="H76" s="123" t="str">
+      <c r="H76" s="124" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F76</f>
         <v>Auteur!D141</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="121" t="n">
+      <c r="A77" s="122" t="n">
         <v>13</v>
       </c>
-      <c r="F77" s="122" t="n">
+      <c r="F77" s="123" t="n">
         <v>142</v>
       </c>
       <c r="G77" s="2" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F77</f>
         <v>Auteur!C142</v>
       </c>
-      <c r="H77" s="123" t="str">
+      <c r="H77" s="124" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F77</f>
         <v>Auteur!D142</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="121" t="n">
+      <c r="A78" s="122" t="n">
         <v>13</v>
       </c>
-      <c r="F78" s="122" t="n">
+      <c r="F78" s="123" t="n">
         <v>143</v>
       </c>
       <c r="G78" s="2" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F78</f>
         <v>Auteur!C143</v>
       </c>
-      <c r="H78" s="123" t="str">
+      <c r="H78" s="124" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F78</f>
         <v>Auteur!D143</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="124" t="n">
+      <c r="A79" s="125" t="n">
         <v>13</v>
       </c>
-      <c r="B79" s="125"/>
-      <c r="C79" s="125"/>
-      <c r="D79" s="125"/>
-      <c r="E79" s="125"/>
-      <c r="F79" s="126" t="n">
+      <c r="B79" s="126"/>
+      <c r="C79" s="126"/>
+      <c r="D79" s="126"/>
+      <c r="E79" s="126"/>
+      <c r="F79" s="127" t="n">
         <v>144</v>
       </c>
-      <c r="G79" s="125" t="str">
+      <c r="G79" s="126" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F79</f>
         <v>Auteur!C144</v>
       </c>
-      <c r="H79" s="127" t="str">
+      <c r="H79" s="128" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F79</f>
         <v>Auteur!D144</v>
       </c>
@@ -8408,7 +8749,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D80</f>
         <v>Auteur!D151</v>
       </c>
-      <c r="F80" s="114" t="n">
+      <c r="F80" s="115" t="n">
         <v>153</v>
       </c>
       <c r="G80" s="2" t="str">
@@ -8592,7 +8933,7 @@
         <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D90</f>
         <v>Auteur!D165</v>
       </c>
-      <c r="F90" s="114" t="n">
+      <c r="F90" s="123" t="n">
         <v>167</v>
       </c>
       <c r="G90" s="2" t="str">
@@ -8602,6 +8943,115 @@
       <c r="H90" s="2" t="str">
         <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F90</f>
         <v>Auteur!D167</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="C91" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;B91</f>
+        <v>Auteur!D169</v>
+      </c>
+      <c r="D91" s="2" t="n">
+        <f aca="false">B91+1</f>
+        <v>170</v>
+      </c>
+      <c r="E91" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$3&amp;D91</f>
+        <v>Auteur!D170</v>
+      </c>
+      <c r="F91" s="123" t="n">
+        <v>172</v>
+      </c>
+      <c r="G91" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F91</f>
+        <v>Auteur!C172</v>
+      </c>
+      <c r="H91" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F91</f>
+        <v>Auteur!D172</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F92" s="123" t="n">
+        <v>173</v>
+      </c>
+      <c r="G92" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F92</f>
+        <v>Auteur!C173</v>
+      </c>
+      <c r="H92" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F92</f>
+        <v>Auteur!D173</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F93" s="123" t="n">
+        <v>174</v>
+      </c>
+      <c r="G93" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F93</f>
+        <v>Auteur!C174</v>
+      </c>
+      <c r="H93" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F93</f>
+        <v>Auteur!D174</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F94" s="123" t="n">
+        <v>175</v>
+      </c>
+      <c r="G94" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F94</f>
+        <v>Auteur!C175</v>
+      </c>
+      <c r="H94" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F94</f>
+        <v>Auteur!D175</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F95" s="123" t="n">
+        <v>176</v>
+      </c>
+      <c r="G95" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F95</f>
+        <v>Auteur!C176</v>
+      </c>
+      <c r="H95" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F95</f>
+        <v>Auteur!D176</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F96" s="123" t="n">
+        <v>177</v>
+      </c>
+      <c r="G96" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F96</f>
+        <v>Auteur!C177</v>
+      </c>
+      <c r="H96" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F96</f>
+        <v>Auteur!D177</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F97" s="123" t="n">
+        <v>178</v>
+      </c>
+      <c r="G97" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$5&amp;F97</f>
+        <v>Auteur!C178</v>
+      </c>
+      <c r="H97" s="2" t="str">
+        <f aca="false">$C$2&amp;"!"&amp;$C$6&amp;F97</f>
+        <v>Auteur!D178</v>
       </c>
     </row>
     <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>